<commit_message>
docs: completar plantilla de requerimientos con estado del prototipo
- Hoja 1: integrante, propósito, alcance, referencias (Guía 11) e
  indicación docente de avanzar sin entrevista.
- Hoja 2: acciones por perfil según la tabla de Guía 10.
- Hoja 3: criterios de aceptación en formato dado/cuando/entonces.
- Hoja 5: dentro y fuera del MVP con fuente; pendientes actualizados.
- Hoja 7: persistencia Room, relaciones y lógica de RN-01/03/05/06.
- Hoja 8: señales de éxito, matriz de trazabilidad y cobertura IE.
- Hoja 9: checklist marcado solo con lo verificado.
Celdas fijas, listas, fórmula y hojas sin cambios.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/entregables/kaiju-requerimientos-guia-10.xlsx
+++ b/docs/entregables/kaiju-requerimientos-guia-10.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="R47c25a26d5d14f76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Introducción y Contexto" sheetId="2" r:id="R61553fe7080d4078"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Roles" sheetId="3" r:id="Re217b9430e5c4223"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Requerimientos (RF)" sheetId="4" r:id="Ra0a158bdcde84bf9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Reglas, RNF y RD" sheetId="5" r:id="R7bd1ebbb10254f35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Alcance" sheetId="6" r:id="Re0eefae40e174037"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Pantallas" sheetId="7" r:id="R7c6803d5851a443b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Modelo de Datos" sheetId="8" r:id="R9695067a95d040d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Trazabilidad" sheetId="9" r:id="R6a90719c359a457c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 Checklist y Aceptación" sheetId="10" r:id="R76dd7d669f4c4d76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="R2a9b091aea8747ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Introducción y Contexto" sheetId="2" r:id="Rdf91b30ab93848a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Roles" sheetId="3" r:id="Rba1383779a704da6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Requerimientos (RF)" sheetId="4" r:id="R80f02a635ac04b19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Reglas, RNF y RD" sheetId="5" r:id="R85d1cd387bfb4c60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Alcance" sheetId="6" r:id="R7a13293f876e4e11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Pantallas" sheetId="7" r:id="Ra5cd6071584f430b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Modelo de Datos" sheetId="8" r:id="R0ae83c7e004f4256"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Trazabilidad" sheetId="9" r:id="R9eeb29bc58464962"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 Checklist y Aceptación" sheetId="10" r:id="R2cccfd09059c432b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -903,95 +903,125 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="6" ht="30" customHeight="1">
+    <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" s="10" t="n"/>
       <x:c r="B6" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Proyecto creado con estructura MVVM (ui, viewmodel, model) y dependencias (Compose, Material 3, Navigation, Room, DataStore).</x:t>
         </x:is>
       </x:c>
-      <x:c r="C6" s="10" t="n"/>
-    </x:row>
-    <x:row r="7" ht="30" customHeight="1">
-      <x:c r="A7" s="10" t="n"/>
+      <x:c r="C6" s="10" t="str">
+        <x:v>Hecho con Room. DataStore no se usa: RD-03 dice Room y/o DataStore.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="48" customHeight="1">
+      <x:c r="A7" s="10" t="str">
+        <x:v>X</x:v>
+      </x:c>
       <x:c r="B7" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Pantalla principal mostrando datos ficticios de prueba en una LazyColumn.</x:t>
         </x:is>
       </x:c>
-      <x:c r="C7" s="10" t="n"/>
-    </x:row>
-    <x:row r="8" ht="30" customHeight="1">
-      <x:c r="A8" s="10" t="n"/>
+      <x:c r="C7" s="10" t="str">
+        <x:v>Catálogo en LazyColumn con 10 productos ficticios.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="48" customHeight="1">
+      <x:c r="A8" s="10" t="str">
+        <x:v>X</x:v>
+      </x:c>
       <x:c r="B8" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Navegación entre pantallas con NavHost.</x:t>
         </x:is>
       </x:c>
-      <x:c r="C8" s="10" t="n"/>
-    </x:row>
-    <x:row r="9" ht="30" customHeight="1">
-      <x:c r="A9" s="10" t="n"/>
+      <x:c r="C8" s="10" t="str">
+        <x:v>Seis rutas con NavHost y menú inferior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="48" customHeight="1">
+      <x:c r="A9" s="10" t="str">
+        <x:v>X</x:v>
+      </x:c>
       <x:c r="B9" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Clases del modelo (hoja 7) creadas como data class, con un ViewModel que expone el estado.</x:t>
         </x:is>
       </x:c>
-      <x:c r="C9" s="10" t="n"/>
-    </x:row>
-    <x:row r="10" ht="30" customHeight="1">
-      <x:c r="A10" s="10" t="n"/>
+      <x:c r="C9" s="10" t="str">
+        <x:v>Producto, Movimiento y Usuario; ViewModels con StateFlow.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="48" customHeight="1">
+      <x:c r="A10" s="10" t="str">
+        <x:v>X</x:v>
+      </x:c>
       <x:c r="B10" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Formularios con validación visual por campo, calculada desde el ViewModel.</x:t>
         </x:is>
       </x:c>
-      <x:c r="C10" s="10" t="n"/>
-    </x:row>
-    <x:row r="11" ht="30" customHeight="1">
-      <x:c r="A11" s="10" t="n"/>
+      <x:c r="C10" s="10" t="str">
+        <x:v>Login, producto y movimiento; 38 pruebas unitarias.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="48" customHeight="1">
+      <x:c r="A11" s="10" t="str">
+        <x:v>X</x:v>
+      </x:c>
       <x:c r="B11" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Reglas de negocio de la hoja 4 implementadas en la capa lógica, no en la interfaz.</x:t>
         </x:is>
       </x:c>
-      <x:c r="C11" s="10" t="n"/>
-    </x:row>
-    <x:row r="12" ht="30" customHeight="1">
+      <x:c r="C11" s="10" t="str">
+        <x:v>RN-01 a RN-06 en InventarioViewModel.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="48" customHeight="1">
       <x:c r="A12" s="10" t="n"/>
       <x:c r="B12" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Persistencia local funcionando (Room y/o DataStore).</x:t>
         </x:is>
       </x:c>
-      <x:c r="C12" s="10" t="n"/>
-    </x:row>
-    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="C12" s="10" t="str">
+        <x:v>Implementado con Room; falta comprobar en teléfono (InventarioDaoTest y pauta paso 19).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="48" customHeight="1">
       <x:c r="A13" s="10" t="n"/>
       <x:c r="B13" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Dos recursos nativos integrados y funcionando sin capturar datos reales de personas.</x:t>
         </x:is>
       </x:c>
-      <x:c r="C13" s="10" t="n"/>
-    </x:row>
-    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="C13" s="10" t="str">
+        <x:v>Notificaciones y lector de códigos implementados; falta probar en teléfono.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="48" customHeight="1">
       <x:c r="A14" s="10" t="n"/>
       <x:c r="B14" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Animaciones que aporten fluidez.</x:t>
         </x:is>
       </x:c>
-      <x:c r="C14" s="10" t="n"/>
-    </x:row>
-    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="C14" s="10" t="str">
+        <x:v>Implementadas; falta revisión visual.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="48" customHeight="1">
       <x:c r="A15" s="10" t="n"/>
       <x:c r="B15" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Repositorio GitHub con commits de todos los integrantes y tablero Trello al día.</x:t>
         </x:is>
       </x:c>
-      <x:c r="C15" s="10" t="n"/>
+      <x:c r="C15" s="10" t="str">
+        <x:v>Commits de un solo integrante (trabajo individual). Sin Trello: consultar al docente.</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="4" t="inlineStr">
@@ -1155,7 +1185,7 @@
         </x:is>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>Integrantes y grupo pendientes. Base académica A-10, versión 07-10-2026. Sin implementación acreditada.</x:v>
+        <x:v>Vicente Hueichapan (trabajo individual). Número de grupo y aceptación docente de la modalidad individual pendientes.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1173,7 +1203,7 @@
         </x:is>
       </x:c>
       <x:c r="B12" s="10" t="str">
-        <x:v>Especificar la base académica de Guía 10 y registrar sus límites, criterios y dudas. No equivale a acta del cliente. Lectura complementaria: docs/11 y docs/12.</x:v>
+        <x:v>Especificar los requerimientos del MVP Kaiju según la base académica de Guía 10 y registrar su estado, origen y pendientes. Lectores: docente, cliente y estudiante. No equivale a acta del cliente: no hubo entrevista.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="60" customHeight="1">
@@ -1183,7 +1213,7 @@
         </x:is>
       </x:c>
       <x:c r="B13" s="10" t="str">
-        <x:v>MVP Kaiju: RF-01 a RF-10 de A-10. Próxima revisión: B-01 a B-09. Persistencia y operación completa se terminan después según §8. Sin ampliar base por ideas opcionales.</x:v>
+        <x:v>App Android Kaiju: consultar existencias, registrar entradas y salidas con historial y detectar stock bajo. Implementa RF-01 a RF-10 de A-10, salvo el alta de producto (G10-02) y el cálculo del ajuste (G10-01). No integra sistemas externos ni usa datos reales. Detalle en hoja 5.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="60" customHeight="1">
@@ -1193,7 +1223,7 @@
         </x:is>
       </x:c>
       <x:c r="B14" s="10" t="str">
-        <x:v>C-01 caso original; N-04 plantilla original; A-10 Guía 10 §1-9, texto proporcionado por usuario; A-10-D1 capas y A-10-D2 navegación, imágenes en docs/fuentes/2026-10-07. Equivalencias históricas en docs/11 §6.</x:v>
+        <x:v>C-01 caso (CITT, 07-09-2026); N-04 plantilla; A-10 Guía 10 §1-9 y diagramas A-10-D1/D2; A-11 Guía 11 (recursos y permisos); guía extra del caso; Cuestionario IEEE 830. Sin acta de entrevista. Repositorio: docs/16 (auditoría) y docs/17 (prototipo).</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1329,7 +1359,7 @@
         </x:is>
       </x:c>
       <x:c r="B31" s="10" t="str">
-        <x:v>Base docente explícita, sin acta comercial. RN-06 y permisos son supuestos revisables declarados en A-10. Pendientes G10-01 a G10-10 en docs/11; navegación parcialmente aclarada por A-10-D2.</x:v>
+        <x:v>Sin acta: la entrevista aún no se agenda. Indicación docente (informada por Vicente el 14-10-2026): avanzar con el material entregado. RN-06 y permisos por perfil son supuestos revisables de A-10 §1. Decisiones técnicas reversibles en docs/17 §1; pendientes G10-01 a G10-10 en docs/11.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1404,7 +1434,7 @@
         <x:v>ADMINISTRADOR en A-10 §4; perfil de prueba.</x:v>
       </x:c>
       <x:c r="C5" s="10" t="str">
-        <x:v>RF-01 a RF-04 y RF-10 comunes; crear/editar, entrada, ajuste y alertas. Permiso para salida pendiente G10-04.</x:v>
+        <x:v>Consulta (RF-01 a RF-04); edita productos (RF-05; crear pendiente G10-02); registra entradas y ajustes (RF-06, RF-08); ve alertas (RF-09). No registra salidas: RF-07 no lo incluye (G10-04).</x:v>
       </x:c>
       <x:c r="D5" s="10" t="str">
         <x:v>Nivel técnico y frecuencia sin información; preguntar P-23.</x:v>
@@ -1420,7 +1450,7 @@
         <x:v>VENDEDOR en A-10 §4; perfil de prueba.</x:v>
       </x:c>
       <x:c r="C6" s="10" t="str">
-        <x:v>RF-01 a RF-04 y RF-10 comunes; salida por venta RF-07. No inferir acceso a ajustes o alertas.</x:v>
+        <x:v>Consulta (RF-01 a RF-04) y registra salidas por venta (RF-07). Sin acceso a alertas, ajustes ni productos.</x:v>
       </x:c>
       <x:c r="D6" s="10" t="str">
         <x:v>Nivel técnico y frecuencia sin información; preguntar P-23.</x:v>
@@ -1436,7 +1466,7 @@
         <x:v>ENCARGADO_INVENTARIO en A-10 §4; perfil de prueba.</x:v>
       </x:c>
       <x:c r="C7" s="10" t="str">
-        <x:v>RF-01 a RF-04 y RF-10 comunes; entradas, salidas, ajustes y alertas. Variantes de salida por aclarar G10-04.</x:v>
+        <x:v>Consulta (RF-01 a RF-04); registra entradas, salidas por venta o consumo y ajustes (RF-06 a RF-08); ve alertas y activa avisos (RF-09).</x:v>
       </x:c>
       <x:c r="D7" s="10" t="str">
         <x:v>Nivel técnico y frecuencia sin información; preguntar P-23.</x:v>
@@ -1568,7 +1598,7 @@
         <x:v>A-10 §1-5, RF-01. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E6" s="10" t="str">
-        <x:v>Sin selección se informa error; con usuario elegido se identifica su perfil. Permisos según tabla docente, con G10-04 aún abierto. Sin contraseñas.</x:v>
+        <x:v>Dado el login sin usuario elegido, cuando se toca Ingresar, entonces se muestra el error y no se ingresa. Dado un usuario elegido, cuando ingresa, entonces se ven su nombre y perfil y solo las acciones de su perfil (tabla A-10 §1).</x:v>
       </x:c>
       <x:c r="F6" s="10" t="str">
         <x:v>1 Login</x:v>
@@ -1590,7 +1620,7 @@
         <x:v>A-10 §1-5, RF-02. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E7" s="10" t="str">
-        <x:v>Con datos ficticios cargados, el catálogo muestra esos cuatro datos desde ViewModel para los tres perfiles base.</x:v>
+        <x:v>Dado el catálogo, cuando lo abre cualquier perfil, entonces cada producto muestra nombre, categoría, precio en CLP y cantidad disponible.</x:v>
       </x:c>
       <x:c r="F7" s="10" t="str">
         <x:v>2 Catálogo</x:v>
@@ -1612,7 +1642,7 @@
         <x:v>A-10 §1-5, RF-03. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E8" s="10" t="str">
-        <x:v>Existen búsqueda y filtro indicados. Casos de coincidencia/combinación pendientes G10-06; no fijar semántica por suposición.</x:v>
+        <x:v>Dado el catálogo, cuando se escribe parte del nombre o del código o se elige una categoría, entonces solo se listan los productos que cumplen ambos criterios. Semántica comercial pendiente G10-06.</x:v>
       </x:c>
       <x:c r="F8" s="10" t="str">
         <x:v>2 Catálogo</x:v>
@@ -1634,7 +1664,7 @@
         <x:v>A-10 §1-5, RF-04. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E9" s="10" t="str">
-        <x:v>Al tocar un producto se abre su detalle e historial asociado, ordenado por fecha descendente. Tipos de fecha/desempate pendientes G10-07.</x:v>
+        <x:v>Dado un producto con movimientos, cuando se abre su detalle, entonces se ven sus datos y su historial (fecha, tipo, cantidad, usuario, motivo) del más reciente al más antiguo.</x:v>
       </x:c>
       <x:c r="F9" s="10" t="str">
         <x:v>3 Detalle</x:v>
@@ -1666,7 +1696,7 @@
         <x:v>A-10 §1-5, RF-05. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
-        <x:v>Código requerido/único; nombre &gt;=3 caracteres; categoría elegida; precio entero &gt;0; mínimo entero &gt;=0. Errores desde VM. Alta visible en catálogo. Stock inicial G10-02 y cambio código G10-03 pendientes.</x:v>
+        <x:v>Dado el administrador, cuando guarda con un campo inválido (A-10 §5), entonces el error aparece en ese campo y no se guarda. Cuando edita con datos válidos, entonces se guardan sin cambiar código ni stock. Alta: valida pero no guarda hasta resolver G10-02.</x:v>
       </x:c>
       <x:c r="F11" s="10" t="str">
         <x:v>4 FormularioProducto</x:v>
@@ -1688,7 +1718,7 @@
         <x:v>A-10 §1-5, RF-06. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E12" s="10" t="str">
-        <x:v>Producto y tipo elegidos, cantidad entera positiva; guardar movimiento y actualizar stock en misma operación. Fecha/autor según RN-05; formato G10-07.</x:v>
+        <x:v>Dado inventario o administrador, cuando registra una entrada con cantidad entera positiva, entonces el disponible aumenta en esa cantidad y el historial suma el movimiento con fecha y usuario, en la misma operación.</x:v>
       </x:c>
       <x:c r="F12" s="10" t="str">
         <x:v>5 Movimiento</x:v>
@@ -1710,7 +1740,7 @@
         <x:v>A-10 §1-5, RF-07. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E13" s="10" t="str">
-        <x:v>Cantidad entera positiva y no superior al stock; una salida válida reduce stock y conserva movimiento en misma operación. Permisos incompletos G10-04.</x:v>
+        <x:v>Dado vendedor (venta) o inventario (venta o consumo), cuando registra una salida no mayor a lo disponible, entonces el disponible baja y queda el movimiento. Si la supera, se muestra el error y nada cambia (RN-01). Permiso del administrador pendiente G10-04.</x:v>
       </x:c>
       <x:c r="F13" s="10" t="str">
         <x:v>5 Movimiento</x:v>
@@ -1732,7 +1762,7 @@
         <x:v>A-10 §1-5, RF-08. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E14" s="10" t="str">
-        <x:v>Sin motivo se informa error. Guardar movimiento/stock juntos con RN-05. Efecto matemático y límites pendientes G10-01; no cerrarlo como implementable.</x:v>
+        <x:v>Dado inventario o administrador, cuando registra un ajuste sin motivo, entonces se muestra el error (RN-04). Efecto sobre el stock pendiente G10-01: con motivo, se informa el pendiente y no se registra.</x:v>
       </x:c>
       <x:c r="F14" s="10" t="str">
         <x:v>5 Movimiento</x:v>
@@ -1764,7 +1794,7 @@
         <x:v>A-10 §1-5, RF-09. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E16" s="10" t="str">
-        <x:v>RN-06: cantidad &lt;= mínimo activa marca y pertenencia a alertas; cantidad &gt; mínimo no. Umbral supuesto docente revisable; no exige notificación del teléfono.</x:v>
+        <x:v>Dado un producto con disponible igual o menor a su mínimo, entonces aparece marcado en el catálogo y en Alertas (inventario y administrador), y al tocarlo se abre su detalle. Si un movimiento lo hace entrar en alerta y hay permiso, llega un aviso al teléfono.</x:v>
       </x:c>
       <x:c r="F16" s="10" t="str">
         <x:v>2 Catálogo; 6 Alertas</x:v>
@@ -1786,7 +1816,7 @@
         <x:v>A-10 §1-5, RF-10. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E17" s="10" t="str">
-        <x:v>Después de guardar cambios, cerrar/reabrir conserva productos e historial. Condición exacta y sesión pendientes G10-08. En memoria no acredita este RF.</x:v>
+        <x:v>Dado un movimiento registrado, cuando se cierra la app y se vuelve a abrir, entonces productos e historial se conservan (Room). La sesión no se conserva: se vuelve a elegir usuario (G10-08).</x:v>
       </x:c>
       <x:c r="F17" s="10" t="str">
         <x:v>Transversal</x:v>
@@ -2504,7 +2534,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="6" ht="100" customHeight="1">
+    <x:row r="6" ht="60" customHeight="1">
       <x:c r="A6" s="10" t="str">
         <x:v>Sesión y consulta</x:v>
       </x:c>
@@ -2515,54 +2545,60 @@
         <x:v>RF-01 a RF-04</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="100" customHeight="1">
+    <x:row r="7" ht="60" customHeight="1">
       <x:c r="A7" s="10" t="str">
         <x:v>Crear y editar productos</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>A-10 RF-05; G10-02/03 limitan criterios todavía abiertos.</x:v>
+        <x:v>Editar implementado (A-10 RF-05). Crear valida, pero no guarda hasta resolver G10-02; código no editable (G10-03).</x:v>
       </x:c>
       <x:c r="C7" s="10" t="str">
         <x:v>RF-05</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="100" customHeight="1">
+    <x:row r="8" ht="60" customHeight="1">
       <x:c r="A8" s="10" t="str">
         <x:v>Entradas, salidas y ajustes</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
-        <x:v>A-10 exige operación; ajuste y algunos permisos requieren precisión.</x:v>
+        <x:v>Entradas y salidas implementadas (A-10 RF-06/07). Ajuste valida el motivo; su efecto espera G10-01.</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
         <x:v>RF-06 a RF-08</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="100" customHeight="1">
+    <x:row r="9" ht="60" customHeight="1">
       <x:c r="A9" s="10" t="str">
-        <x:v>Alertas dentro de app</x:v>
+        <x:v>Alertas, marca de stock bajo y aviso del teléfono</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>A-10 RN-06 y RF-09; umbral revisable.</x:v>
+        <x:v>A-10 RN-06 y RF-09; aviso por notificación según C-01 §3.3 y RD-04. Umbral revisable.</x:v>
       </x:c>
       <x:c r="C9" s="10" t="str">
         <x:v>RF-09</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="100" customHeight="1">
+    <x:row r="10" ht="60" customHeight="1">
       <x:c r="A10" s="10" t="str">
         <x:v>Conservación local</x:v>
       </x:c>
       <x:c r="B10" s="10" t="str">
-        <x:v>Exigencia final A-10; memoria primero según §3/8.</x:v>
+        <x:v>Implementado con Room (RD-03). La sesión no se guarda (G10-08).</x:v>
       </x:c>
       <x:c r="C10" s="10" t="str">
         <x:v>RF-10</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="24" customHeight="1">
-      <x:c r="A11" s="10" t="n"/>
-      <x:c r="B11" s="10" t="n"/>
-      <x:c r="C11" s="10" t="n"/>
+    <x:row r="11" ht="60" customHeight="1">
+      <x:c r="A11" s="10" t="str">
+        <x:v>Lector de códigos para elegir el producto</x:v>
+      </x:c>
+      <x:c r="B11" s="10" t="str">
+        <x:v>C-01 §3.3 menciona la cámara para leer códigos; cumple RD-04 junto con las notificaciones. Sin permiso de cámara.</x:v>
+      </x:c>
+      <x:c r="C11" s="10" t="str">
+        <x:v>RF-06, RF-07</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="4" t="inlineStr">
@@ -2596,15 +2632,27 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="15" ht="24" customHeight="1">
-      <x:c r="A15" s="10" t="n"/>
-      <x:c r="B15" s="10" t="n"/>
-      <x:c r="C15" s="10" t="n"/>
-    </x:row>
-    <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="10" t="n"/>
-      <x:c r="B16" s="10" t="n"/>
-      <x:c r="C16" s="10" t="n"/>
+    <x:row r="15" ht="45" customHeight="1">
+      <x:c r="A15" s="10" t="str">
+        <x:v>Integración con sistemas de venta, catálogos digitales o facturación</x:v>
+      </x:c>
+      <x:c r="B15" s="10" t="str">
+        <x:v>C-01 §3.4 y §5.1: no se exige para el MVP; se considera deseable a futuro.</x:v>
+      </x:c>
+      <x:c r="C15" s="10" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="45" customHeight="1">
+      <x:c r="A16" s="10" t="str">
+        <x:v>Uso de datos reales, credenciales o accesos de Kaiju</x:v>
+      </x:c>
+      <x:c r="B16" s="10" t="str">
+        <x:v>Prohibido por C-01 §5.1 y RD-05: solo datos ficticios.</x:v>
+      </x:c>
+      <x:c r="C16" s="10" t="str">
+        <x:v>No</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="10" t="n"/>
@@ -2709,15 +2757,15 @@
         <x:v>Por acordar; no inventar fechas.</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="100" customHeight="1">
+    <x:row r="27" ht="70" customHeight="1">
       <x:c r="A27" s="10" t="str">
-        <x:v>Equipo y decisiones propias</x:v>
+        <x:v>Equipo, evaluación y módulo propio</x:v>
       </x:c>
       <x:c r="B27" s="10" t="str">
-        <x:v>Integrantes/grupo, recursos, animaciones, módulo e identidad aún no elegidos.</x:v>
+        <x:v>Aceptación del trabajo individual y evidencia sin Trello (IE 2.3.2). Módulo propio: más/menos vendidos o tendencias (C-01 §4.1) requieren medida y período (P-13, P-14).</x:v>
       </x:c>
       <x:c r="C27" s="10" t="str">
-        <x:v>Equipo; docente valida evaluación.</x:v>
+        <x:v>Docente (evaluación); cliente (módulo).</x:v>
       </x:c>
       <x:c r="D27" s="10" t="str">
         <x:v>Por acordar; no inventar fechas.</x:v>
@@ -2869,7 +2917,7 @@
         <x:v>Administrador (A-10 §2; A-10-D2).</x:v>
       </x:c>
       <x:c r="D8" s="10" t="str">
-        <x:v>Botón + del Catálogo, según A-10-D2; entrada a edición por precisar (A-10 §2; A-10-D2).</x:v>
+        <x:v>Botón + del Catálogo (crear) y botón Editar en el detalle (A-10 §2; A-10-D2).</x:v>
       </x:c>
       <x:c r="E8" s="10" t="str">
         <x:v>Validaciones §5. Stock inicial/código editable pendientes G10-02/03. (A-10 §2; A-10-D2).</x:v>
@@ -2892,7 +2940,7 @@
         <x:v>Menú inferior; registrar desde detalle (A-10 §2; A-10-D2).</x:v>
       </x:c>
       <x:c r="E9" s="10" t="str">
-        <x:v>Producto/tipo/cantidad, motivo en ajuste. Fórmula pendiente G10-01. (A-10 §2; A-10-D2).</x:v>
+        <x:v>Producto (lista o lector de códigos), tipo según perfil, cantidad entera positiva, motivo obligatorio en ajuste. Fórmula del ajuste pendiente G10-01. (A-10 §2, §5)</x:v>
       </x:c>
       <x:c r="F9" s="10" t="str">
         <x:v>RF-06/07/08 (A-10 §2; A-10-D2).</x:v>
@@ -2912,7 +2960,7 @@
         <x:v>Menú inferior; variación por perfil por precisar (A-10 §2; A-10-D2).</x:v>
       </x:c>
       <x:c r="E10" s="10" t="str">
-        <x:v>Lista bajo mínimo; tocar abre detalle. No notificación nativa exigida aquí. (A-10 §2; A-10-D2).</x:v>
+        <x:v>Lista bajo mínimo; tocar abre detalle. Tarjeta para activar avisos con permiso POST_NOTIFICATIONS (A-11 §4). (A-10 §2)</x:v>
       </x:c>
       <x:c r="F10" s="10" t="str">
         <x:v>RF-09 (A-10 §2; A-10-D2).</x:v>
@@ -3016,31 +3064,35 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="5" ht="100" customHeight="1">
+    <x:row r="5" ht="75" customHeight="1">
       <x:c r="A5" s="10" t="str">
         <x:v>Producto</x:v>
       </x:c>
       <x:c r="B5" s="10" t="str">
         <x:v>codigo, nombre, descripcion, categoria, tipo, precio Int CLP, stockActual, stockMinimo, detalle opcional texto. Otros tipos pendientes. A-10 §4.</x:v>
       </x:c>
-      <x:c r="C5" s="10" t="n"/>
+      <x:c r="C5" s="10" t="str">
+        <x:v>Room</x:v>
+      </x:c>
       <x:c r="D5" s="10" t="str">
-        <x:v>Movimiento usa codigoProducto. Política de cambio código G10-03. Memoria ahora; persistencia por decidir después.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="100" customHeight="1">
+        <x:v>Clave primaria: codigo. Un producto tiene muchos movimientos. stockActual solo cambia al registrar un movimiento (A-10 §4).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="75" customHeight="1">
       <x:c r="A6" s="10" t="str">
         <x:v>Movimiento</x:v>
       </x:c>
       <x:c r="B6" s="10" t="str">
         <x:v>id, codigoProducto, tipo (enum), cantidad, motivo, fecha, usuario. Tipos/políticas pendientes G10-07. A-10 §4.</x:v>
       </x:c>
-      <x:c r="C6" s="10" t="n"/>
+      <x:c r="C6" s="10" t="str">
+        <x:v>Room</x:v>
+      </x:c>
       <x:c r="D6" s="10" t="str">
-        <x:v>Vinculado a producto y autor; no editar/borrar. Ajuste pendiente G10-01. Memoria ahora; persistencia por decidir después.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="100" customHeight="1">
+        <x:v>codigoProducto es clave foránea a Producto. No se edita ni se borra (RN-05). Se guarda junto con el stock en una transacción.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="75" customHeight="1">
       <x:c r="A7" s="10" t="str">
         <x:v>Usuario</x:v>
       </x:c>
@@ -3049,7 +3101,7 @@
       </x:c>
       <x:c r="C7" s="10" t="n"/>
       <x:c r="D7" s="10" t="str">
-        <x:v>Autor del movimiento y selección de sesión; representación por precisar. Memoria ahora; persistencia por decidir después.</x:v>
+        <x:v>Autor del movimiento (se copia en él). Los tres usuarios de prueba viven en el código y no se guardan; la sesión tampoco (G10-08).</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="100" customHeight="1">
@@ -3070,21 +3122,33 @@
       <x:c r="C9" s="10" t="n"/>
       <x:c r="D9" s="10" t="n"/>
     </x:row>
-    <x:row r="10" ht="24" customHeight="1">
-      <x:c r="A10" s="10" t="n"/>
-      <x:c r="B10" s="10" t="n"/>
+    <x:row r="10" ht="110" customHeight="1">
+      <x:c r="A10" s="10" t="str">
+        <x:v>Lógica: registrar una salida (RN-01, RN-05)</x:v>
+      </x:c>
+      <x:c r="B10" s="10" t="str">
+        <x:v>1) ¿Hay producto y tipo elegidos y el perfil puede usar ese tipo? 2) ¿La cantidad es entera y mayor que cero? 3) ¿La cantidad es menor o igual al disponible? Si algo falla: error en su campo, no se guarda. Si todo está bien: disponible − cantidad y movimiento con fecha y usuario, en una sola transacción.</x:v>
+      </x:c>
       <x:c r="C10" s="10" t="n"/>
       <x:c r="D10" s="10" t="n"/>
     </x:row>
-    <x:row r="11" ht="24" customHeight="1">
-      <x:c r="A11" s="10" t="n"/>
-      <x:c r="B11" s="10" t="n"/>
+    <x:row r="11" ht="110" customHeight="1">
+      <x:c r="A11" s="10" t="str">
+        <x:v>Lógica: alerta de stock (RN-06)</x:v>
+      </x:c>
+      <x:c r="B11" s="10" t="str">
+        <x:v>Un producto está en alerta si stockActual &lt;= stockMinimo. La misma función marca el catálogo, arma la lista de Alertas y decide el aviso: solo se notifica cuando un movimiento hace pasar el producto de no estar en alerta a estarlo.</x:v>
+      </x:c>
       <x:c r="C11" s="10" t="n"/>
       <x:c r="D11" s="10" t="n"/>
     </x:row>
-    <x:row r="12" ht="24" customHeight="1">
-      <x:c r="A12" s="10" t="n"/>
-      <x:c r="B12" s="10" t="n"/>
+    <x:row r="12" ht="110" customHeight="1">
+      <x:c r="A12" s="10" t="str">
+        <x:v>Lógica: código de producto (RN-03)</x:v>
+      </x:c>
+      <x:c r="B12" s="10" t="str">
+        <x:v>Al crear: código sin espacios al inicio ni al final; si está vacío o ya existe, error y no se guarda. Al editar, el código no cambia porque identifica el historial (G10-03).</x:v>
+      </x:c>
       <x:c r="C12" s="10" t="n"/>
       <x:c r="D12" s="10" t="n"/>
     </x:row>
@@ -3177,73 +3241,85 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="6" ht="30" customHeight="1">
+    <x:row r="6" ht="45" customHeight="1">
       <x:c r="A6" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Stock actualizado y trazable por producto.</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" s="10" t="n"/>
+      <x:c r="B6" s="10" t="str">
+        <x:v>RF-02, RF-04, RF-06, RF-07, RF-10 y RN-05: stock visible, historial con fecha y autor, stock y movimiento guardados juntos.</x:v>
+      </x:c>
       <x:c r="C6" s="12" t="n"/>
       <x:c r="D6" s="12" t="n"/>
       <x:c r="E6" s="12" t="n"/>
       <x:c r="F6" s="11" t="n"/>
     </x:row>
-    <x:row r="7" ht="30" customHeight="1">
+    <x:row r="7" ht="45" customHeight="1">
       <x:c r="A7" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Disminución de quiebres de stock y diferencias de inventario.</x:t>
         </x:is>
       </x:c>
-      <x:c r="B7" s="10" t="n"/>
+      <x:c r="B7" s="10" t="str">
+        <x:v>RF-09 y RN-06 (alertas y aviso), RN-01 (sin stock negativo), RF-08 ajuste con motivo (efecto pendiente G10-01). Sin métrica acordada para medir la disminución (P-18).</x:v>
+      </x:c>
       <x:c r="C7" s="12" t="n"/>
       <x:c r="D7" s="12" t="n"/>
       <x:c r="E7" s="12" t="n"/>
       <x:c r="F7" s="11" t="n"/>
     </x:row>
-    <x:row r="8" ht="30" customHeight="1">
+    <x:row r="8" ht="45" customHeight="1">
       <x:c r="A8" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Identificación rápida de productos más vendidos y menos vendidos.</x:t>
         </x:is>
       </x:c>
-      <x:c r="B8" s="10" t="n"/>
+      <x:c r="B8" s="10" t="str">
+        <x:v>Sin cobertura todavía: candidato a módulo propio desde RF-11; requiere P-13.</x:v>
+      </x:c>
       <x:c r="C8" s="12" t="n"/>
       <x:c r="D8" s="12" t="n"/>
       <x:c r="E8" s="12" t="n"/>
       <x:c r="F8" s="11" t="n"/>
     </x:row>
-    <x:row r="9" ht="30" customHeight="1">
+    <x:row r="9" ht="45" customHeight="1">
       <x:c r="A9" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Visualización de tendencias de venta por período, categoría o tipo de producto.</x:t>
         </x:is>
       </x:c>
-      <x:c r="B9" s="10" t="n"/>
+      <x:c r="B9" s="10" t="str">
+        <x:v>Sin cobertura todavía: candidato a módulo propio; requiere P-14.</x:v>
+      </x:c>
       <x:c r="C9" s="12" t="n"/>
       <x:c r="D9" s="12" t="n"/>
       <x:c r="E9" s="12" t="n"/>
       <x:c r="F9" s="11" t="n"/>
     </x:row>
-    <x:row r="10" ht="30" customHeight="1">
+    <x:row r="10" ht="45" customHeight="1">
       <x:c r="A10" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Mayor rapidez en el registro de entradas, salidas y ventas.</x:t>
         </x:is>
       </x:c>
-      <x:c r="B10" s="10" t="n"/>
+      <x:c r="B10" s="10" t="str">
+        <x:v>RF-06 y RF-07 con lector de códigos y formulario que conserva producto y tipo. Sin métrica acordada (P-25).</x:v>
+      </x:c>
       <x:c r="C10" s="12" t="n"/>
       <x:c r="D10" s="12" t="n"/>
       <x:c r="E10" s="12" t="n"/>
       <x:c r="F10" s="11" t="n"/>
     </x:row>
-    <x:row r="11" ht="30" customHeight="1">
+    <x:row r="11" ht="45" customHeight="1">
       <x:c r="A11" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Información de disponibilidad más clara para usuarios internos y público general.</x:t>
         </x:is>
       </x:c>
-      <x:c r="B11" s="10" t="n"/>
+      <x:c r="B11" s="10" t="str">
+        <x:v>Interna: RF-02 y RF-03. Público general condicional (C-01 §3.1), no incluido; pendiente P-05.</x:v>
+      </x:c>
       <x:c r="C11" s="12" t="n"/>
       <x:c r="D11" s="12" t="n"/>
       <x:c r="E11" s="12" t="n"/>
@@ -3293,85 +3369,205 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="15" ht="20" customHeight="1">
-      <x:c r="A15" s="10" t="n"/>
-      <x:c r="B15" s="10" t="n"/>
-      <x:c r="C15" s="10" t="n"/>
-      <x:c r="D15" s="10" t="n"/>
-      <x:c r="E15" s="10" t="n"/>
-      <x:c r="F15" s="10" t="n"/>
-    </x:row>
-    <x:row r="16" ht="20" customHeight="1">
-      <x:c r="A16" s="10" t="n"/>
-      <x:c r="B16" s="10" t="n"/>
-      <x:c r="C16" s="10" t="n"/>
-      <x:c r="D16" s="10" t="n"/>
-      <x:c r="E16" s="10" t="n"/>
-      <x:c r="F16" s="10" t="n"/>
-    </x:row>
-    <x:row r="17" ht="20" customHeight="1">
-      <x:c r="A17" s="10" t="n"/>
-      <x:c r="B17" s="10" t="n"/>
-      <x:c r="C17" s="10" t="n"/>
-      <x:c r="D17" s="10" t="n"/>
-      <x:c r="E17" s="10" t="n"/>
-      <x:c r="F17" s="10" t="n"/>
-    </x:row>
-    <x:row r="18" ht="20" customHeight="1">
-      <x:c r="A18" s="10" t="n"/>
-      <x:c r="B18" s="10" t="n"/>
-      <x:c r="C18" s="10" t="n"/>
-      <x:c r="D18" s="10" t="n"/>
-      <x:c r="E18" s="10" t="n"/>
-      <x:c r="F18" s="10" t="n"/>
-    </x:row>
-    <x:row r="19" ht="20" customHeight="1">
-      <x:c r="A19" s="10" t="n"/>
-      <x:c r="B19" s="10" t="n"/>
-      <x:c r="C19" s="10" t="n"/>
-      <x:c r="D19" s="10" t="n"/>
-      <x:c r="E19" s="10" t="n"/>
-      <x:c r="F19" s="10" t="n"/>
-    </x:row>
-    <x:row r="20" ht="20" customHeight="1">
-      <x:c r="A20" s="10" t="n"/>
-      <x:c r="B20" s="10" t="n"/>
-      <x:c r="C20" s="10" t="n"/>
-      <x:c r="D20" s="10" t="n"/>
-      <x:c r="E20" s="10" t="n"/>
-      <x:c r="F20" s="10" t="n"/>
-    </x:row>
-    <x:row r="21" ht="20" customHeight="1">
-      <x:c r="A21" s="10" t="n"/>
-      <x:c r="B21" s="10" t="n"/>
-      <x:c r="C21" s="10" t="n"/>
-      <x:c r="D21" s="10" t="n"/>
-      <x:c r="E21" s="10" t="n"/>
-      <x:c r="F21" s="10" t="n"/>
-    </x:row>
-    <x:row r="22" ht="20" customHeight="1">
-      <x:c r="A22" s="10" t="n"/>
-      <x:c r="B22" s="10" t="n"/>
-      <x:c r="C22" s="10" t="n"/>
-      <x:c r="D22" s="10" t="n"/>
-      <x:c r="E22" s="10" t="n"/>
-      <x:c r="F22" s="10" t="n"/>
-    </x:row>
-    <x:row r="23" ht="20" customHeight="1">
-      <x:c r="A23" s="10" t="n"/>
-      <x:c r="B23" s="10" t="n"/>
-      <x:c r="C23" s="10" t="n"/>
-      <x:c r="D23" s="10" t="n"/>
-      <x:c r="E23" s="10" t="n"/>
-      <x:c r="F23" s="10" t="n"/>
-    </x:row>
-    <x:row r="24" ht="20" customHeight="1">
-      <x:c r="A24" s="10" t="n"/>
-      <x:c r="B24" s="10" t="n"/>
-      <x:c r="C24" s="10" t="n"/>
-      <x:c r="D24" s="10" t="n"/>
-      <x:c r="E24" s="10" t="n"/>
-      <x:c r="F24" s="10" t="n"/>
+    <x:row r="15" ht="45" customHeight="1">
+      <x:c r="A15" s="10" t="str">
+        <x:v>RF-01</x:v>
+      </x:c>
+      <x:c r="B15" s="10" t="str">
+        <x:v>A-10 §1</x:v>
+      </x:c>
+      <x:c r="C15" s="10" t="str">
+        <x:v>1 Login</x:v>
+      </x:c>
+      <x:c r="D15" s="10" t="str">
+        <x:v>SesionViewModel; AppNavHost</x:v>
+      </x:c>
+      <x:c r="E15" s="10" t="str">
+        <x:v>SesionViewModelTest (4 pruebas)</x:v>
+      </x:c>
+      <x:c r="F15" s="10" t="str">
+        <x:v>IE 2.1.1, IE 2.1.2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="45" customHeight="1">
+      <x:c r="A16" s="10" t="str">
+        <x:v>RF-02</x:v>
+      </x:c>
+      <x:c r="B16" s="10" t="str">
+        <x:v>A-10 §1</x:v>
+      </x:c>
+      <x:c r="C16" s="10" t="str">
+        <x:v>2 Catálogo</x:v>
+      </x:c>
+      <x:c r="D16" s="10" t="str">
+        <x:v>InventarioViewModel.catalogo; TarjetaProducto</x:v>
+      </x:c>
+      <x:c r="E16" s="10" t="str">
+        <x:v>catalogoMuestraLosDiezProductosDePrueba</x:v>
+      </x:c>
+      <x:c r="F16" s="10" t="str">
+        <x:v>IE 2.1.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="45" customHeight="1">
+      <x:c r="A17" s="10" t="str">
+        <x:v>RF-03</x:v>
+      </x:c>
+      <x:c r="B17" s="10" t="str">
+        <x:v>A-10 §1</x:v>
+      </x:c>
+      <x:c r="C17" s="10" t="str">
+        <x:v>2 Catálogo</x:v>
+      </x:c>
+      <x:c r="D17" s="10" t="str">
+        <x:v>InventarioViewModel.filtro y catalogo</x:v>
+      </x:c>
+      <x:c r="E17" s="10" t="str">
+        <x:v>buscaPorNombreOCodigoParcial...; filtroPorCategoriaSeCombina...</x:v>
+      </x:c>
+      <x:c r="F17" s="10" t="str">
+        <x:v>IE 2.1.1, IE 2.2.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="45" customHeight="1">
+      <x:c r="A18" s="10" t="str">
+        <x:v>RF-04</x:v>
+      </x:c>
+      <x:c r="B18" s="10" t="str">
+        <x:v>A-10 §1-2</x:v>
+      </x:c>
+      <x:c r="C18" s="10" t="str">
+        <x:v>3 Detalle</x:v>
+      </x:c>
+      <x:c r="D18" s="10" t="str">
+        <x:v>InventarioViewModel.historial</x:v>
+      </x:c>
+      <x:c r="E18" s="10" t="str">
+        <x:v>historialDelMasRecienteAlMasAntiguo...</x:v>
+      </x:c>
+      <x:c r="F18" s="10" t="str">
+        <x:v>IE 2.1.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="45" customHeight="1">
+      <x:c r="A19" s="10" t="str">
+        <x:v>RF-05</x:v>
+      </x:c>
+      <x:c r="B19" s="10" t="str">
+        <x:v>A-10 §1, §5</x:v>
+      </x:c>
+      <x:c r="C19" s="10" t="str">
+        <x:v>4 Formulario producto</x:v>
+      </x:c>
+      <x:c r="D19" s="10" t="str">
+        <x:v>InventarioViewModel.validarProducto y guardarProducto</x:v>
+      </x:c>
+      <x:c r="E19" s="10" t="str">
+        <x:v>InventarioViewModelTest (validación, edición y permisos)</x:v>
+      </x:c>
+      <x:c r="F19" s="10" t="str">
+        <x:v>IE 2.1.2, IE 2.2.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="45" customHeight="1">
+      <x:c r="A20" s="10" t="str">
+        <x:v>RF-06</x:v>
+      </x:c>
+      <x:c r="B20" s="10" t="str">
+        <x:v>A-10 §1, §4</x:v>
+      </x:c>
+      <x:c r="C20" s="10" t="str">
+        <x:v>5 Movimiento</x:v>
+      </x:c>
+      <x:c r="D20" s="10" t="str">
+        <x:v>InventarioViewModel.registrarMovimiento; InventarioDao</x:v>
+      </x:c>
+      <x:c r="E20" s="10" t="str">
+        <x:v>entradaSumaStock...; InventarioDaoTest (en teléfono)</x:v>
+      </x:c>
+      <x:c r="F20" s="10" t="str">
+        <x:v>IE 2.1.2, IE 2.2.1, IE 2.3.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="45" customHeight="1">
+      <x:c r="A21" s="10" t="str">
+        <x:v>RF-07</x:v>
+      </x:c>
+      <x:c r="B21" s="10" t="str">
+        <x:v>A-10 §1, RN-01</x:v>
+      </x:c>
+      <x:c r="C21" s="10" t="str">
+        <x:v>5 Movimiento</x:v>
+      </x:c>
+      <x:c r="D21" s="10" t="str">
+        <x:v>InventarioViewModel.validarMovimiento</x:v>
+      </x:c>
+      <x:c r="E21" s="10" t="str">
+        <x:v>ventaIgualALoDisponible...; salidaMayorALoDisponible...</x:v>
+      </x:c>
+      <x:c r="F21" s="10" t="str">
+        <x:v>IE 2.2.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="45" customHeight="1">
+      <x:c r="A22" s="10" t="str">
+        <x:v>RF-08</x:v>
+      </x:c>
+      <x:c r="B22" s="10" t="str">
+        <x:v>A-10 §1, RN-04</x:v>
+      </x:c>
+      <x:c r="C22" s="10" t="str">
+        <x:v>5 Movimiento</x:v>
+      </x:c>
+      <x:c r="D22" s="10" t="str">
+        <x:v>InventarioViewModel.validarMovimiento</x:v>
+      </x:c>
+      <x:c r="E22" s="10" t="str">
+        <x:v>ajusteSinMotivoSeRechaza; ajusteValidoNoCambiaStock...</x:v>
+      </x:c>
+      <x:c r="F22" s="10" t="str">
+        <x:v>IE 2.2.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="45" customHeight="1">
+      <x:c r="A23" s="10" t="str">
+        <x:v>RF-09</x:v>
+      </x:c>
+      <x:c r="B23" s="10" t="str">
+        <x:v>A-10 §1, RN-06; C-01 §3.3</x:v>
+      </x:c>
+      <x:c r="C23" s="10" t="str">
+        <x:v>2 Catálogo; 6 Alertas</x:v>
+      </x:c>
+      <x:c r="D23" s="10" t="str">
+        <x:v>estaEnAlerta; alertas; NotificacionesStock</x:v>
+      </x:c>
+      <x:c r="E23" s="10" t="str">
+        <x:v>igualdadConMinimoEstaEnAlerta; avisaSoloCuando...; pauta docs/17</x:v>
+      </x:c>
+      <x:c r="F23" s="10" t="str">
+        <x:v>IE 2.1.1, IE 2.2.2, IE 2.4.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="45" customHeight="1">
+      <x:c r="A24" s="10" t="str">
+        <x:v>RF-10</x:v>
+      </x:c>
+      <x:c r="B24" s="10" t="str">
+        <x:v>A-10 §1; RD-03</x:v>
+      </x:c>
+      <x:c r="C24" s="10" t="str">
+        <x:v>Transversal</x:v>
+      </x:c>
+      <x:c r="D24" s="10" t="str">
+        <x:v>BaseDeDatosKaiju; InventarioRepositoryRoom</x:v>
+      </x:c>
+      <x:c r="E24" s="10" t="str">
+        <x:v>InventarioDaoTest (en teléfono); pauta docs/17 paso 19</x:v>
+      </x:c>
+      <x:c r="F24" s="10" t="str">
+        <x:v>IE 2.3.1</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="20" customHeight="1">
       <x:c r="A25" s="10" t="n"/>
@@ -3433,7 +3629,7 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="30" ht="20" customHeight="1">
+    <x:row r="30" ht="35" customHeight="1">
       <x:c r="A30" s="7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">IE 2.1.1</x:t>
@@ -3447,11 +3643,13 @@
       <x:c r="C30" s="8" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="D30" s="10" t="n"/>
+      <x:c r="D30" s="10" t="str">
+        <x:v>RF-01 a RF-04 y RF-09: seis pantallas, menú inferior e identidad visual.</x:v>
+      </x:c>
       <x:c r="E30" s="12" t="n"/>
       <x:c r="F30" s="11" t="n"/>
     </x:row>
-    <x:row r="31" ht="20" customHeight="1">
+    <x:row r="31" ht="35" customHeight="1">
       <x:c r="A31" s="7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">IE 2.1.2</x:t>
@@ -3465,11 +3663,13 @@
       <x:c r="C31" s="8" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="D31" s="10" t="n"/>
+      <x:c r="D31" s="10" t="str">
+        <x:v>RF-01, RF-05, RF-06 a RF-08: formularios de login, producto y movimiento con error e ícono por campo.</x:v>
+      </x:c>
       <x:c r="E31" s="12" t="n"/>
       <x:c r="F31" s="11" t="n"/>
     </x:row>
-    <x:row r="32" ht="20" customHeight="1">
+    <x:row r="32" ht="35" customHeight="1">
       <x:c r="A32" s="7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">IE 2.2.1</x:t>
@@ -3483,11 +3683,13 @@
       <x:c r="C32" s="8" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="D32" s="10" t="n"/>
+      <x:c r="D32" s="10" t="str">
+        <x:v>RN-01 a RN-06 en InventarioViewModel, antes de llamar al repositorio.</x:v>
+      </x:c>
       <x:c r="E32" s="12" t="n"/>
       <x:c r="F32" s="11" t="n"/>
     </x:row>
-    <x:row r="33" ht="20" customHeight="1">
+    <x:row r="33" ht="35" customHeight="1">
       <x:c r="A33" s="7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">IE 2.2.2</x:t>
@@ -3501,11 +3703,13 @@
       <x:c r="C33" s="8" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="D33" s="10" t="n"/>
+      <x:c r="D33" s="10" t="str">
+        <x:v>RF-09: marca de stock bajo animada y color del disponible; confirmación con Snackbar.</x:v>
+      </x:c>
       <x:c r="E33" s="12" t="n"/>
       <x:c r="F33" s="11" t="n"/>
     </x:row>
-    <x:row r="34" ht="20" customHeight="1">
+    <x:row r="34" ht="35" customHeight="1">
       <x:c r="A34" s="7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">IE 2.3.1</x:t>
@@ -3519,11 +3723,13 @@
       <x:c r="C34" s="8" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="D34" s="10" t="n"/>
+      <x:c r="D34" s="10" t="str">
+        <x:v>RF-10, RD-02 y RD-03: capas separadas y Room detrás del repositorio.</x:v>
+      </x:c>
       <x:c r="E34" s="12" t="n"/>
       <x:c r="F34" s="11" t="n"/>
     </x:row>
-    <x:row r="35" ht="20" customHeight="1">
+    <x:row r="35" ht="35" customHeight="1">
       <x:c r="A35" s="7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">IE 2.3.2</x:t>
@@ -3545,7 +3751,7 @@
       <x:c r="E35" s="12" t="n"/>
       <x:c r="F35" s="11" t="n"/>
     </x:row>
-    <x:row r="36" ht="20" customHeight="1">
+    <x:row r="36" ht="35" customHeight="1">
       <x:c r="A36" s="7" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">IE 2.4.1</x:t>
@@ -3559,7 +3765,9 @@
       <x:c r="C36" s="8" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="D36" s="10" t="n"/>
+      <x:c r="D36" s="10" t="str">
+        <x:v>RD-04: notificaciones de stock bajo (RF-09) y lector de códigos (RF-06, RF-07).</x:v>
+      </x:c>
       <x:c r="E36" s="12" t="n"/>
       <x:c r="F36" s="11" t="n"/>
     </x:row>

</xml_diff>

<commit_message>
feat: persistencia local con Room según la guía y el ejemplo docente
- database/: BaseDeDatosKaiju (singleton obtenerInstancia) e InventarioDao.
- repository/InventarioRepository: clase que envuelve al DAO, único que lo conoce.
- viewmodel/InventarioViewModelFactory, usada por AppNavHost.
- Pruebas con FakeInventarioDao (como FakeEventoDao) y PersistenciaViewModelTest
  que simula reabrir la app; 40 pruebas aprobadas.
- Investigación §10 comentada en el código: @ForeignKey y migraciones (esquema).
- Guía de Room guardada como fuente; documentación y evidencia actualizadas.
</commit_message>
<xml_diff>
--- a/docs/entregables/kaiju-requerimientos-guia-10.xlsx
+++ b/docs/entregables/kaiju-requerimientos-guia-10.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="R2a9b091aea8747ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Introducción y Contexto" sheetId="2" r:id="Rdf91b30ab93848a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Roles" sheetId="3" r:id="Rba1383779a704da6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Requerimientos (RF)" sheetId="4" r:id="R80f02a635ac04b19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Reglas, RNF y RD" sheetId="5" r:id="R85d1cd387bfb4c60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Alcance" sheetId="6" r:id="R7a13293f876e4e11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Pantallas" sheetId="7" r:id="Ra5cd6071584f430b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Modelo de Datos" sheetId="8" r:id="R0ae83c7e004f4256"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Trazabilidad" sheetId="9" r:id="R9eeb29bc58464962"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 Checklist y Aceptación" sheetId="10" r:id="R2cccfd09059c432b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="Rcfdde051af7b4b5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Introducción y Contexto" sheetId="2" r:id="Re4c715eb11cd415a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Roles" sheetId="3" r:id="R6a49c86f5a5a4a06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Requerimientos (RF)" sheetId="4" r:id="R77dd051a2bf84926"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Reglas, RNF y RD" sheetId="5" r:id="Rc9cda29d58cc4705"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Alcance" sheetId="6" r:id="Rb2cf77a7def74b6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Pantallas" sheetId="7" r:id="R3a150acd58654b3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Modelo de Datos" sheetId="8" r:id="R709f3e2e1c2e4cf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Trazabilidad" sheetId="9" r:id="R6b0148d014f84784"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 Checklist y Aceptación" sheetId="10" r:id="Rdaef51e4806b4ccc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -963,7 +963,7 @@
         </x:is>
       </x:c>
       <x:c r="C10" s="10" t="str">
-        <x:v>Login, producto y movimiento; 38 pruebas unitarias.</x:v>
+        <x:v>Login, producto y movimiento; 40 pruebas unitarias.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -3560,10 +3560,10 @@
         <x:v>Transversal</x:v>
       </x:c>
       <x:c r="D24" s="10" t="str">
-        <x:v>BaseDeDatosKaiju; InventarioRepositoryRoom</x:v>
+        <x:v>database/BaseDeDatosKaiju e InventarioDao; InventarioRepository; InventarioViewModelFactory</x:v>
       </x:c>
       <x:c r="E24" s="10" t="str">
-        <x:v>InventarioDaoTest (en teléfono); pauta docs/17 paso 19</x:v>
+        <x:v>PersistenciaViewModelTest (reabrir); InventarioDaoTest (en teléfono); pauta docs/17 paso 19</x:v>
       </x:c>
       <x:c r="F24" s="10" t="str">
         <x:v>IE 2.3.1</x:v>

</xml_diff>

<commit_message>
docs: escribir sección en vez de § y ordenar evidencia del código
- Se reemplaza el símbolo § por la palabra sección en código, documentos y plantilla (las fuentes originales no se modifican).
- En el código y la documentación vigente se usan nombres legibles (Guía 10, Guía 11, caso) en vez de códigos internos.
- docs/evidencia/CODIGO.md: cada archivo por capa, con su propósito, requisito y prueba.
- Word de evidencia regenerado. 40 pruebas aprobadas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/entregables/kaiju-requerimientos-guia-10.xlsx
+++ b/docs/entregables/kaiju-requerimientos-guia-10.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="Rcfdde051af7b4b5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Introducción y Contexto" sheetId="2" r:id="Re4c715eb11cd415a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Roles" sheetId="3" r:id="R6a49c86f5a5a4a06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Requerimientos (RF)" sheetId="4" r:id="R77dd051a2bf84926"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Reglas, RNF y RD" sheetId="5" r:id="Rc9cda29d58cc4705"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Alcance" sheetId="6" r:id="Rb2cf77a7def74b6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Pantallas" sheetId="7" r:id="R3a150acd58654b3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Modelo de Datos" sheetId="8" r:id="R709f3e2e1c2e4cf6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Trazabilidad" sheetId="9" r:id="R6b0148d014f84784"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 Checklist y Aceptación" sheetId="10" r:id="Rdaef51e4806b4ccc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="R2cac95139fe34a7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Introducción y Contexto" sheetId="2" r:id="Ra73f52cd9cca474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Roles" sheetId="3" r:id="R31525bace67a4008"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Requerimientos (RF)" sheetId="4" r:id="R6298d405a6b543bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Reglas, RNF y RD" sheetId="5" r:id="R197603a205384f48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Alcance" sheetId="6" r:id="R46e2d1b0b8544fdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Pantallas" sheetId="7" r:id="R1ddf37e9bcf141b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Modelo de Datos" sheetId="8" r:id="R3f9694f0a4dd4a3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Trazabilidad" sheetId="9" r:id="Rd577b521bfa34cc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 Checklist y Aceptación" sheetId="10" r:id="R68e54f1f87014294"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1213,7 +1213,7 @@
         </x:is>
       </x:c>
       <x:c r="B13" s="10" t="str">
-        <x:v>App Android Kaiju: consultar existencias, registrar entradas y salidas con historial y detectar stock bajo. Implementa RF-01 a RF-10 de A-10, salvo el alta de producto (G10-02) y el cálculo del ajuste (G10-01). No integra sistemas externos ni usa datos reales. Detalle en hoja 5.</x:v>
+        <x:v>App Android Kaiju: consultar existencias, registrar entradas y salidas con historial y detectar stock bajo. Implementa RF-01 a RF-10 de Guía 10, salvo el alta de producto (G10-02) y el cálculo del ajuste (G10-01). No integra sistemas externos ni usa datos reales. Detalle en hoja 5.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="60" customHeight="1">
@@ -1223,7 +1223,7 @@
         </x:is>
       </x:c>
       <x:c r="B14" s="10" t="str">
-        <x:v>C-01 caso (CITT, 07-09-2026); N-04 plantilla; A-10 Guía 10 §1-9 y diagramas A-10-D1/D2; A-11 Guía 11 (recursos y permisos); guía extra del caso; Cuestionario IEEE 830. Sin acta de entrevista. Repositorio: docs/16 (auditoría) y docs/17 (prototipo).</x:v>
+        <x:v>Caso Kaiju (CITT, 07-09-2026); plantilla de requerimientos; Guía 10 (secciones 1 a 9) y sus diagramas de capas y navegación; Guía 11 (recursos y permisos); guía de persistencia con Room; guía extra del caso; Cuestionario IEEE 830. Sin acta de entrevista. Repositorio: docs/16 (auditoría) y docs/17 (prototipo).</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1251,7 +1251,7 @@
         <x:v>Producto</x:v>
       </x:c>
       <x:c r="B18" s="10" t="str">
-        <x:v>Definición documental provisional, no acordada: Artículo sobre el que se registran datos, cantidades y movimientos; C-01 §2.1/§3.2. Pendiente: Relación con materiales/insumos y atributos; P-06, P-07.</x:v>
+        <x:v>Definición documental provisional, no acordada: Artículo sobre el que se registran datos, cantidades y movimientos; caso sección 2.1/sección 3.2. Pendiente: Relación con materiales/insumos y atributos; P-06, P-07.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="60" customHeight="1">
@@ -1259,7 +1259,7 @@
         <x:v>Existencia / stock</x:v>
       </x:c>
       <x:c r="B19" s="10" t="str">
-        <x:v>Base A-10 §4-5: stockActual representa cantidad disponible; unidades reales y stock inicial al crear siguen pendientes G10-02. No acordado con cliente.</x:v>
+        <x:v>Base Guía 10 sección 4-5: stockActual representa cantidad disponible; unidades reales y stock inicial al crear siguen pendientes G10-02. No acordado con cliente.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="60" customHeight="1">
@@ -1267,7 +1267,7 @@
         <x:v>Movimiento</x:v>
       </x:c>
       <x:c r="B20" s="10" t="str">
-        <x:v>Base A-10 §4: ENTRADA, SALIDA_VENTA, SALIDA_CONSUMO y AJUSTE; guarda datos RN-05. Forma del ajuste pendiente G10-01. No acta comercial.</x:v>
+        <x:v>Base Guía 10 sección 4: ENTRADA, SALIDA_VENTA, SALIDA_CONSUMO y AJUSTE; guarda datos RN-05. Forma del ajuste pendiente G10-01. No acta comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="60" customHeight="1">
@@ -1275,7 +1275,7 @@
         <x:v>Venta</x:v>
       </x:c>
       <x:c r="B21" s="10" t="str">
-        <x:v>Base A-10 RF-07: salida por venta; no confirma documento comercial completo. C-01 menciona ventas. Composición adicional pendiente P-10.</x:v>
+        <x:v>Base Guía 10 RF-07: salida por venta; no confirma documento comercial completo. caso menciona ventas. Composición adicional pendiente P-10.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="60" customHeight="1">
@@ -1283,7 +1283,7 @@
         <x:v>Stock mínimo</x:v>
       </x:c>
       <x:c r="B22" s="10" t="str">
-        <x:v>Base A-10 RN-06: alerta si stockActual &lt;= stockMinimo. Umbral supuesto revisable del profesor; no validación comercial.</x:v>
+        <x:v>Base Guía 10 RN-06: alerta si stockActual &lt;= stockMinimo. Umbral supuesto revisable del profesor; no validación comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="60" customHeight="1">
@@ -1291,7 +1291,7 @@
         <x:v>Trazabilidad</x:v>
       </x:c>
       <x:c r="B23" s="10" t="str">
-        <x:v>Base A-10 RN-05: historial con fecha/tipo/cantidad/autor; no editar ni borrar movimientos, corregir mediante ajuste. Cliente aún sin validar.</x:v>
+        <x:v>Base Guía 10 RN-05: historial con fecha/tipo/cantidad/autor; no editar ni borrar movimientos, corregir mediante ajuste. Cliente aún sin validar.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1309,7 +1309,7 @@
         </x:is>
       </x:c>
       <x:c r="B26" s="10" t="str">
-        <x:v>Kaiju recibe, almacena, utiliza o vende productos, materiales e insumos. Hoy usa registros manuales y planillas que requieren actualización. C-01 §2.1-2.2.</x:v>
+        <x:v>Kaiju recibe, almacena, utiliza o vende productos, materiales e insumos. Hoy usa registros manuales y planillas que requieren actualización. caso sección 2.1-2.2.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="60" customHeight="1">
@@ -1319,7 +1319,7 @@
         </x:is>
       </x:c>
       <x:c r="B27" s="10" t="str">
-        <x:v>Posibles diferencias de existencias, movimientos omitidos y detección tardía de reposición dificultan el control y las decisiones. No hay mediciones aportadas. C-01 §2.3.</x:v>
+        <x:v>Posibles diferencias de existencias, movimientos omitidos y detección tardía de reposición dificultan el control y las decisiones. No hay mediciones aportadas. caso sección 2.3.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="60" customHeight="1">
@@ -1329,7 +1329,7 @@
         </x:is>
       </x:c>
       <x:c r="B28" s="10" t="str">
-        <x:v>Facilitar consulta y registro/revisión de movimientos para mejorar control y trazabilidad. Rapidez, actualización y mejora requieren criterios acordados. C-01 §2.4 y §4.1; P-11, P-15, P-18.</x:v>
+        <x:v>Facilitar consulta y registro/revisión de movimientos para mejorar control y trazabilidad. Rapidez, actualización y mejora requieren criterios acordados. caso sección 2.4 y sección 4.1; P-11, P-15, P-18.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="60" customHeight="1">
@@ -1339,7 +1339,7 @@
         </x:is>
       </x:c>
       <x:c r="B29" s="10" t="str">
-        <x:v>MVP Android académico. Integración con sistemas existentes no exigida; conexiones futuras deseables. RD académicas en hoja 4. C-01 §3.3-3.4 y §5.1.</x:v>
+        <x:v>MVP Android académico. Integración con sistemas existentes no exigida; conexiones futuras deseables. RD académicas en hoja 4. caso sección 3.3-3.4 y sección 5.1.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="60" customHeight="1">
@@ -1349,7 +1349,7 @@
         </x:is>
       </x:c>
       <x:c r="B30" s="10" t="str">
-        <x:v>Material académico autorizado: datos ficticios, sintéticos, agregados, públicos o anonimizados. Sin datos personales reales, registros productivos, accesos internos ni credenciales de Kaiju. C-01 §5.1; RD-05.</x:v>
+        <x:v>Material académico autorizado: datos ficticios, sintéticos, agregados, públicos o anonimizados. Sin datos personales reales, registros productivos, accesos internos ni credenciales de Kaiju. caso sección 5.1; RD-05.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="60" customHeight="1">
@@ -1359,7 +1359,7 @@
         </x:is>
       </x:c>
       <x:c r="B31" s="10" t="str">
-        <x:v>Sin acta: la entrevista aún no se agenda. Indicación docente (informada por Vicente el 14-10-2026): avanzar con el material entregado. RN-06 y permisos por perfil son supuestos revisables de A-10 §1. Decisiones técnicas reversibles en docs/17 §1; pendientes G10-01 a G10-10 en docs/11.</x:v>
+        <x:v>Sin acta: la entrevista aún no se agenda. Indicación docente (informada por Vicente el 14-10-2026): avanzar con el material entregado. RN-06 y permisos por perfil son supuestos revisables de Guía 10 sección 1. Decisiones técnicas reversibles en docs/17 sección 1; pendientes G10-01 a G10-10 en docs/11.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1431,7 +1431,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="10" t="str">
-        <x:v>ADMINISTRADOR en A-10 §4; perfil de prueba.</x:v>
+        <x:v>ADMINISTRADOR en Guía 10 sección 4; perfil de prueba.</x:v>
       </x:c>
       <x:c r="C5" s="10" t="str">
         <x:v>Consulta (RF-01 a RF-04); edita productos (RF-05; crear pendiente G10-02); registra entradas y ajustes (RF-06, RF-08); ve alertas (RF-09). No registra salidas: RF-07 no lo incluye (G10-04).</x:v>
@@ -1447,7 +1447,7 @@
         </x:is>
       </x:c>
       <x:c r="B6" s="10" t="str">
-        <x:v>VENDEDOR en A-10 §4; perfil de prueba.</x:v>
+        <x:v>VENDEDOR en Guía 10 sección 4; perfil de prueba.</x:v>
       </x:c>
       <x:c r="C6" s="10" t="str">
         <x:v>Consulta (RF-01 a RF-04) y registra salidas por venta (RF-07). Sin acceso a alertas, ajustes ni productos.</x:v>
@@ -1463,7 +1463,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>ENCARGADO_INVENTARIO en A-10 §4; perfil de prueba.</x:v>
+        <x:v>ENCARGADO_INVENTARIO en Guía 10 sección 4; perfil de prueba.</x:v>
       </x:c>
       <x:c r="C7" s="10" t="str">
         <x:v>Consulta (RF-01 a RF-04); registra entradas, salidas por venta o consumo y ajustes (RF-06 a RF-08); ve alertas y activa avisos (RF-09).</x:v>
@@ -1479,7 +1479,7 @@
         </x:is>
       </x:c>
       <x:c r="B8" s="10" t="str">
-        <x:v>Condicional en C-01; no es uno de los tres perfiles de la base A-10.</x:v>
+        <x:v>Condicional en caso; no es uno de los tres perfiles de la base Guía 10.</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
         <x:v>Consulta pública no incorporada automáticamente. Mantener P-05 y módulo propio pendiente.</x:v>
@@ -1595,10 +1595,10 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D6" s="10" t="str">
-        <x:v>A-10 §1-5, RF-01. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-01. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E6" s="10" t="str">
-        <x:v>Dado el login sin usuario elegido, cuando se toca Ingresar, entonces se muestra el error y no se ingresa. Dado un usuario elegido, cuando ingresa, entonces se ven su nombre y perfil y solo las acciones de su perfil (tabla A-10 §1).</x:v>
+        <x:v>Dado el login sin usuario elegido, cuando se toca Ingresar, entonces se muestra el error y no se ingresa. Dado un usuario elegido, cuando ingresa, entonces se ven su nombre y perfil y solo las acciones de su perfil (tabla Guía 10 sección 1).</x:v>
       </x:c>
       <x:c r="F6" s="10" t="str">
         <x:v>1 Login</x:v>
@@ -1617,7 +1617,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D7" s="10" t="str">
-        <x:v>A-10 §1-5, RF-02. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-02. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E7" s="10" t="str">
         <x:v>Dado el catálogo, cuando lo abre cualquier perfil, entonces cada producto muestra nombre, categoría, precio en CLP y cantidad disponible.</x:v>
@@ -1639,7 +1639,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D8" s="10" t="str">
-        <x:v>A-10 §1-5, RF-03. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-03. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E8" s="10" t="str">
         <x:v>Dado el catálogo, cuando se escribe parte del nombre o del código o se elige una categoría, entonces solo se listan los productos que cumplen ambos criterios. Semántica comercial pendiente G10-06.</x:v>
@@ -1661,7 +1661,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
-        <x:v>A-10 §1-5, RF-04. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-04. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E9" s="10" t="str">
         <x:v>Dado un producto con movimientos, cuando se abre su detalle, entonces se ven sus datos y su historial (fecha, tipo, cantidad, usuario, motivo) del más reciente al más antiguo.</x:v>
@@ -1693,10 +1693,10 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
-        <x:v>A-10 §1-5, RF-05. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-05. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
-        <x:v>Dado el administrador, cuando guarda con un campo inválido (A-10 §5), entonces el error aparece en ese campo y no se guarda. Cuando edita con datos válidos, entonces se guardan sin cambiar código ni stock. Alta: valida pero no guarda hasta resolver G10-02.</x:v>
+        <x:v>Dado el administrador, cuando guarda con un campo inválido (Guía 10 sección 5), entonces el error aparece en ese campo y no se guarda. Cuando edita con datos válidos, entonces se guardan sin cambiar código ni stock. Alta: valida pero no guarda hasta resolver G10-02.</x:v>
       </x:c>
       <x:c r="F11" s="10" t="str">
         <x:v>4 FormularioProducto</x:v>
@@ -1715,7 +1715,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D12" s="10" t="str">
-        <x:v>A-10 §1-5, RF-06. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-06. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E12" s="10" t="str">
         <x:v>Dado inventario o administrador, cuando registra una entrada con cantidad entera positiva, entonces el disponible aumenta en esa cantidad y el historial suma el movimiento con fecha y usuario, en la misma operación.</x:v>
@@ -1737,7 +1737,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D13" s="10" t="str">
-        <x:v>A-10 §1-5, RF-07. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-07. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E13" s="10" t="str">
         <x:v>Dado vendedor (venta) o inventario (venta o consumo), cuando registra una salida no mayor a lo disponible, entonces el disponible baja y queda el movimiento. Si la supera, se muestra el error y nada cambia (RN-01). Permiso del administrador pendiente G10-04.</x:v>
@@ -1759,7 +1759,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D14" s="10" t="str">
-        <x:v>A-10 §1-5, RF-08. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-08. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E14" s="10" t="str">
         <x:v>Dado inventario o administrador, cuando registra un ajuste sin motivo, entonces se muestra el error (RN-04). Efecto sobre el stock pendiente G10-01: con motivo, se informa el pendiente y no se registra.</x:v>
@@ -1791,7 +1791,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D16" s="10" t="str">
-        <x:v>A-10 §1-5, RF-09. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-09. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E16" s="10" t="str">
         <x:v>Dado un producto con disponible igual o menor a su mínimo, entonces aparece marcado en el catálogo y en Alertas (inventario y administrador), y al tocarlo se abre su detalle. Si un movimiento lo hace entrar en alerta y hay permiso, llega un aviso al teléfono.</x:v>
@@ -1813,7 +1813,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D17" s="10" t="str">
-        <x:v>A-10 §1-5, RF-10. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-10. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E17" s="10" t="str">
         <x:v>Dado un movimiento registrado, cuando se cierra la app y se vuelve a abrir, entonces productos e historial se conservan (Room). La sesión no se conserva: se vuelve a elegir usuario (G10-08).</x:v>
@@ -2016,7 +2016,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="F6" s="10" t="str">
-        <x:v>A-10 §1; §4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
+        <x:v>Guía 10 sección 1; sección 4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="100" customHeight="1">
@@ -2029,7 +2029,7 @@
         <x:v>Precio y mínimo</x:v>
       </x:c>
       <x:c r="C7" s="10" t="str">
-        <x:v>Precio &gt;0 y stock mínimo &gt;=0. A-10 §4-5 exige enteros, precio en CLP.</x:v>
+        <x:v>Precio &gt;0 y stock mínimo &gt;=0. Guía 10 sección 4-5 exige enteros, precio en CLP.</x:v>
       </x:c>
       <x:c r="D7" s="10" t="str">
         <x:v>Precio 1 y mínimo 0 cumplen; precio 0 o mínimo -1 no cumplen.</x:v>
@@ -2038,7 +2038,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="F7" s="10" t="str">
-        <x:v>A-10 §1; §4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
+        <x:v>Guía 10 sección 1; sección 4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="100" customHeight="1">
@@ -2060,7 +2060,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="F8" s="10" t="str">
-        <x:v>A-10 §1; §4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
+        <x:v>Guía 10 sección 1; sección 4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="100" customHeight="1">
@@ -2082,7 +2082,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="F9" s="10" t="str">
-        <x:v>A-10 §1; §4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
+        <x:v>Guía 10 sección 1; sección 4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="100" customHeight="1">
@@ -2104,7 +2104,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="F10" s="10" t="str">
-        <x:v>A-10 §1; §4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
+        <x:v>Guía 10 sección 1; sección 4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="100" customHeight="1">
@@ -2126,7 +2126,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="F11" s="10" t="str">
-        <x:v>A-10 §1; §4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
+        <x:v>Guía 10 sección 1; sección 4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2188,7 +2188,7 @@
       </x:c>
       <x:c r="E15" s="10" t="n"/>
       <x:c r="F15" s="10" t="str">
-        <x:v>C-01 §4.1; RNF-01 candidato. Categoría y prioridad pendientes.</x:v>
+        <x:v>caso sección 4.1; RNF-01 candidato. Categoría y prioridad pendientes.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="100" customHeight="1">
@@ -2206,7 +2206,7 @@
       </x:c>
       <x:c r="E16" s="10" t="n"/>
       <x:c r="F16" s="10" t="str">
-        <x:v>C-01 §4.1 y §3.3; RNF-02 candidato. Categoría y prioridad pendientes.</x:v>
+        <x:v>caso sección 4.1 y sección 3.3; RNF-02 candidato. Categoría y prioridad pendientes.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="100" customHeight="1">
@@ -2224,7 +2224,7 @@
       </x:c>
       <x:c r="E17" s="10" t="n"/>
       <x:c r="F17" s="10" t="str">
-        <x:v>C-01 §3.3; RNF-03 candidato. Categoría y prioridad pendientes.</x:v>
+        <x:v>caso sección 3.3; RNF-03 candidato. Categoría y prioridad pendientes.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
@@ -2539,7 +2539,7 @@
         <x:v>Sesión y consulta</x:v>
       </x:c>
       <x:c r="B6" s="10" t="str">
-        <x:v>RF-01 a RF-04: explícitos A-10; no autenticación productiva.</x:v>
+        <x:v>RF-01 a RF-04: explícitos Guía 10; no autenticación productiva.</x:v>
       </x:c>
       <x:c r="C6" s="10" t="str">
         <x:v>RF-01 a RF-04</x:v>
@@ -2550,7 +2550,7 @@
         <x:v>Crear y editar productos</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>Editar implementado (A-10 RF-05). Crear valida, pero no guarda hasta resolver G10-02; código no editable (G10-03).</x:v>
+        <x:v>Editar implementado (Guía 10 RF-05). Crear valida, pero no guarda hasta resolver G10-02; código no editable (G10-03).</x:v>
       </x:c>
       <x:c r="C7" s="10" t="str">
         <x:v>RF-05</x:v>
@@ -2561,7 +2561,7 @@
         <x:v>Entradas, salidas y ajustes</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
-        <x:v>Entradas y salidas implementadas (A-10 RF-06/07). Ajuste valida el motivo; su efecto espera G10-01.</x:v>
+        <x:v>Entradas y salidas implementadas (Guía 10 RF-06/07). Ajuste valida el motivo; su efecto espera G10-01.</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
         <x:v>RF-06 a RF-08</x:v>
@@ -2572,7 +2572,7 @@
         <x:v>Alertas, marca de stock bajo y aviso del teléfono</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>A-10 RN-06 y RF-09; aviso por notificación según C-01 §3.3 y RD-04. Umbral revisable.</x:v>
+        <x:v>Guía 10 RN-06 y RF-09; aviso por notificación según caso sección 3.3 y RD-04. Umbral revisable.</x:v>
       </x:c>
       <x:c r="C9" s="10" t="str">
         <x:v>RF-09</x:v>
@@ -2594,7 +2594,7 @@
         <x:v>Lector de códigos para elegir el producto</x:v>
       </x:c>
       <x:c r="B11" s="10" t="str">
-        <x:v>C-01 §3.3 menciona la cámara para leer códigos; cumple RD-04 junto con las notificaciones. Sin permiso de cámara.</x:v>
+        <x:v>caso sección 3.3 menciona la cámara para leer códigos; cumple RD-04 junto con las notificaciones. Sin permiso de cámara.</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
         <x:v>RF-06, RF-07</x:v>
@@ -2637,7 +2637,7 @@
         <x:v>Integración con sistemas de venta, catálogos digitales o facturación</x:v>
       </x:c>
       <x:c r="B15" s="10" t="str">
-        <x:v>C-01 §3.4 y §5.1: no se exige para el MVP; se considera deseable a futuro.</x:v>
+        <x:v>caso sección 3.4 y sección 5.1: no se exige para el MVP; se considera deseable a futuro.</x:v>
       </x:c>
       <x:c r="C15" s="10" t="str">
         <x:v>Sí</x:v>
@@ -2648,7 +2648,7 @@
         <x:v>Uso de datos reales, credenciales o accesos de Kaiju</x:v>
       </x:c>
       <x:c r="B16" s="10" t="str">
-        <x:v>Prohibido por C-01 §5.1 y RD-05: solo datos ficticios.</x:v>
+        <x:v>Prohibido por caso sección 5.1 y RD-05: solo datos ficticios.</x:v>
       </x:c>
       <x:c r="C16" s="10" t="str">
         <x:v>No</x:v>
@@ -2720,7 +2720,7 @@
         <x:v>Navegación y permisos</x:v>
       </x:c>
       <x:c r="B24" s="10" t="str">
-        <x:v>Destinos resueltos A-10-D2; variación por rol y algunas salidas pendientes G10-04.</x:v>
+        <x:v>Destinos resueltos diagrama 2 de la Guía 10; variación por rol y algunas salidas pendientes G10-04.</x:v>
       </x:c>
       <x:c r="C24" s="10" t="str">
         <x:v>Docente / cliente según validación.</x:v>
@@ -2762,7 +2762,7 @@
         <x:v>Equipo, evaluación y módulo propio</x:v>
       </x:c>
       <x:c r="B27" s="10" t="str">
-        <x:v>Aceptación del trabajo individual y evidencia sin Trello (IE 2.3.2). Módulo propio: más/menos vendidos o tendencias (C-01 §4.1) requieren medida y período (P-13, P-14).</x:v>
+        <x:v>Aceptación del trabajo individual y evidencia sin Trello (IE 2.3.2). Módulo propio: más/menos vendidos o tendencias (caso sección 4.1) requieren medida y período (P-13, P-14).</x:v>
       </x:c>
       <x:c r="C27" s="10" t="str">
         <x:v>Docente (evaluación); cliente (módulo).</x:v>
@@ -2851,19 +2851,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B5" s="10" t="str">
-        <x:v>PantallaLogin (A-10 §2; A-10-D2).</x:v>
+        <x:v>PantallaLogin (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="C5" s="10" t="str">
-        <x:v>Tres usuarios de prueba (A-10 §2; A-10-D2).</x:v>
+        <x:v>Tres usuarios de prueba (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="D5" s="10" t="str">
-        <x:v>Entrada de app (A-10 §2; A-10-D2).</x:v>
+        <x:v>Entrada de app (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="E5" s="10" t="str">
-        <x:v>Elegir usuario obligatorio, error desde SesionViewModel. (A-10 §2; A-10-D2).</x:v>
+        <x:v>Elegir usuario obligatorio, error desde SesionViewModel. (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="F5" s="10" t="str">
-        <x:v>RF-01 (A-10 §2; A-10-D2).</x:v>
+        <x:v>RF-01 (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="100" customHeight="1">
@@ -2871,19 +2871,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="10" t="str">
-        <x:v>PantallaCatalogo (A-10 §2; A-10-D2).</x:v>
+        <x:v>PantallaCatalogo (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="C6" s="10" t="str">
-        <x:v>Tres perfiles base (A-10 §2; A-10-D2).</x:v>
+        <x:v>Tres perfiles base (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="D6" s="10" t="str">
-        <x:v>Login; menú inferior (A-10 §2; A-10-D2).</x:v>
+        <x:v>Login; menú inferior (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="E6" s="10" t="str">
-        <x:v>Nombre/categoría/precio/cantidad, búsqueda/filtro, marca bajo mínimo. (A-10 §2; A-10-D2).</x:v>
+        <x:v>Nombre/categoría/precio/cantidad, búsqueda/filtro, marca bajo mínimo. (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="F6" s="10" t="str">
-        <x:v>RF-02/03/09 (A-10 §2; A-10-D2).</x:v>
+        <x:v>RF-02/03/09 (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="100" customHeight="1">
@@ -2891,19 +2891,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>PantallaDetalleProducto (A-10 §2; A-10-D2).</x:v>
+        <x:v>PantallaDetalleProducto (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="C7" s="10" t="str">
-        <x:v>Tres perfiles base (A-10 §2; A-10-D2).</x:v>
+        <x:v>Tres perfiles base (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="D7" s="10" t="str">
-        <x:v>Catálogo al tocar producto; alerta al tocarla (A-10 §2; A-10-D2).</x:v>
+        <x:v>Catálogo al tocar producto; alerta al tocarla (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="E7" s="10" t="str">
-        <x:v>Datos e historial por producto, recientes primero. (A-10 §2; A-10-D2).</x:v>
+        <x:v>Datos e historial por producto, recientes primero. (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="F7" s="10" t="str">
-        <x:v>RF-04 (A-10 §2; A-10-D2).</x:v>
+        <x:v>RF-04 (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="100" customHeight="1">
@@ -2911,19 +2911,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
-        <x:v>PantallaFormularioProducto (A-10 §2; A-10-D2).</x:v>
+        <x:v>PantallaFormularioProducto (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
-        <x:v>Administrador (A-10 §2; A-10-D2).</x:v>
+        <x:v>Administrador (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="D8" s="10" t="str">
-        <x:v>Botón + del Catálogo (crear) y botón Editar en el detalle (A-10 §2; A-10-D2).</x:v>
+        <x:v>Botón + del Catálogo (crear) y botón Editar en el detalle (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="E8" s="10" t="str">
-        <x:v>Validaciones §5. Stock inicial/código editable pendientes G10-02/03. (A-10 §2; A-10-D2).</x:v>
+        <x:v>Validaciones sección 5. Stock inicial/código editable pendientes G10-02/03. (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="F8" s="10" t="str">
-        <x:v>RF-05 (A-10 §2; A-10-D2).</x:v>
+        <x:v>RF-05 (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="100" customHeight="1">
@@ -2931,19 +2931,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>PantallaMovimiento (A-10 §2; A-10-D2).</x:v>
+        <x:v>PantallaMovimiento (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="C9" s="10" t="str">
-        <x:v>Según perfil y tipo; permisos G10-04 (A-10 §2; A-10-D2).</x:v>
+        <x:v>Según perfil y tipo; permisos G10-04 (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
-        <x:v>Menú inferior; registrar desde detalle (A-10 §2; A-10-D2).</x:v>
+        <x:v>Menú inferior; registrar desde detalle (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="E9" s="10" t="str">
-        <x:v>Producto (lista o lector de códigos), tipo según perfil, cantidad entera positiva, motivo obligatorio en ajuste. Fórmula del ajuste pendiente G10-01. (A-10 §2, §5)</x:v>
+        <x:v>Producto (lista o lector de códigos), tipo según perfil, cantidad entera positiva, motivo obligatorio en ajuste. Fórmula del ajuste pendiente G10-01. (Guía 10 sección 2, sección 5)</x:v>
       </x:c>
       <x:c r="F9" s="10" t="str">
-        <x:v>RF-06/07/08 (A-10 §2; A-10-D2).</x:v>
+        <x:v>RF-06/07/08 (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="100" customHeight="1">
@@ -2951,19 +2951,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B10" s="10" t="str">
-        <x:v>PantallaAlertas (A-10 §2; A-10-D2).</x:v>
+        <x:v>PantallaAlertas (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="C10" s="10" t="str">
-        <x:v>Inventario y administrador (A-10 §2; A-10-D2).</x:v>
+        <x:v>Inventario y administrador (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="D10" s="10" t="str">
-        <x:v>Menú inferior; variación por perfil por precisar (A-10 §2; A-10-D2).</x:v>
+        <x:v>Menú inferior; variación por perfil por precisar (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="E10" s="10" t="str">
-        <x:v>Lista bajo mínimo; tocar abre detalle. Tarjeta para activar avisos con permiso POST_NOTIFICATIONS (A-11 §4). (A-10 §2)</x:v>
+        <x:v>Lista bajo mínimo; tocar abre detalle. Tarjeta para activar avisos con permiso POST_NOTIFICATIONS (Guía 11 sección 4). (Guía 10 sección 2)</x:v>
       </x:c>
       <x:c r="F10" s="10" t="str">
-        <x:v>RF-09 (A-10 §2; A-10-D2).</x:v>
+        <x:v>RF-09 (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
@@ -3069,13 +3069,13 @@
         <x:v>Producto</x:v>
       </x:c>
       <x:c r="B5" s="10" t="str">
-        <x:v>codigo, nombre, descripcion, categoria, tipo, precio Int CLP, stockActual, stockMinimo, detalle opcional texto. Otros tipos pendientes. A-10 §4.</x:v>
+        <x:v>codigo, nombre, descripcion, categoria, tipo, precio Int CLP, stockActual, stockMinimo, detalle opcional texto. Otros tipos pendientes. Guía 10 sección 4.</x:v>
       </x:c>
       <x:c r="C5" s="10" t="str">
         <x:v>Room</x:v>
       </x:c>
       <x:c r="D5" s="10" t="str">
-        <x:v>Clave primaria: codigo. Un producto tiene muchos movimientos. stockActual solo cambia al registrar un movimiento (A-10 §4).</x:v>
+        <x:v>Clave primaria: codigo. Un producto tiene muchos movimientos. stockActual solo cambia al registrar un movimiento (Guía 10 sección 4).</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="75" customHeight="1">
@@ -3083,7 +3083,7 @@
         <x:v>Movimiento</x:v>
       </x:c>
       <x:c r="B6" s="10" t="str">
-        <x:v>id, codigoProducto, tipo (enum), cantidad, motivo, fecha, usuario. Tipos/políticas pendientes G10-07. A-10 §4.</x:v>
+        <x:v>id, codigoProducto, tipo (enum), cantidad, motivo, fecha, usuario. Tipos/políticas pendientes G10-07. Guía 10 sección 4.</x:v>
       </x:c>
       <x:c r="C6" s="10" t="str">
         <x:v>Room</x:v>
@@ -3097,7 +3097,7 @@
         <x:v>Usuario</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>id, nombre, rol (enum). Tres usuarios ficticios; no personas reales. A-10 §4.</x:v>
+        <x:v>id, nombre, rol (enum). Tres usuarios ficticios; no personas reales. Guía 10 sección 4.</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n"/>
       <x:c r="D7" s="10" t="str">
@@ -3109,11 +3109,11 @@
         <x:v>Enums</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
-        <x:v>TipoMovimiento: ENTRADA, SALIDA_VENTA, SALIDA_CONSUMO, AJUSTE. Rol: ADMINISTRADOR, VENDEDOR, ENCARGADO_INVENTARIO. A-10 §4.</x:v>
+        <x:v>TipoMovimiento: ENTRADA, SALIDA_VENTA, SALIDA_CONSUMO, AJUSTE. Rol: ADMINISTRADOR, VENDEDOR, ENCARGADO_INVENTARIO. Guía 10 sección 4.</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n"/>
       <x:c r="D8" s="10" t="str">
-        <x:v>A-10 §4. No son tablas obligatorias independientes. Memoria ahora; persistencia por decidir después.</x:v>
+        <x:v>Guía 10 sección 4. No son tablas obligatorias independientes. Memoria ahora; persistencia por decidir después.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
@@ -3318,7 +3318,7 @@
         </x:is>
       </x:c>
       <x:c r="B11" s="10" t="str">
-        <x:v>Interna: RF-02 y RF-03. Público general condicional (C-01 §3.1), no incluido; pendiente P-05.</x:v>
+        <x:v>Interna: RF-02 y RF-03. Público general condicional (caso sección 3.1), no incluido; pendiente P-05.</x:v>
       </x:c>
       <x:c r="C11" s="12" t="n"/>
       <x:c r="D11" s="12" t="n"/>
@@ -3374,7 +3374,7 @@
         <x:v>RF-01</x:v>
       </x:c>
       <x:c r="B15" s="10" t="str">
-        <x:v>A-10 §1</x:v>
+        <x:v>Guía 10 sección 1</x:v>
       </x:c>
       <x:c r="C15" s="10" t="str">
         <x:v>1 Login</x:v>
@@ -3394,7 +3394,7 @@
         <x:v>RF-02</x:v>
       </x:c>
       <x:c r="B16" s="10" t="str">
-        <x:v>A-10 §1</x:v>
+        <x:v>Guía 10 sección 1</x:v>
       </x:c>
       <x:c r="C16" s="10" t="str">
         <x:v>2 Catálogo</x:v>
@@ -3414,7 +3414,7 @@
         <x:v>RF-03</x:v>
       </x:c>
       <x:c r="B17" s="10" t="str">
-        <x:v>A-10 §1</x:v>
+        <x:v>Guía 10 sección 1</x:v>
       </x:c>
       <x:c r="C17" s="10" t="str">
         <x:v>2 Catálogo</x:v>
@@ -3434,7 +3434,7 @@
         <x:v>RF-04</x:v>
       </x:c>
       <x:c r="B18" s="10" t="str">
-        <x:v>A-10 §1-2</x:v>
+        <x:v>Guía 10 sección 1-2</x:v>
       </x:c>
       <x:c r="C18" s="10" t="str">
         <x:v>3 Detalle</x:v>
@@ -3454,7 +3454,7 @@
         <x:v>RF-05</x:v>
       </x:c>
       <x:c r="B19" s="10" t="str">
-        <x:v>A-10 §1, §5</x:v>
+        <x:v>Guía 10 sección 1, sección 5</x:v>
       </x:c>
       <x:c r="C19" s="10" t="str">
         <x:v>4 Formulario producto</x:v>
@@ -3474,7 +3474,7 @@
         <x:v>RF-06</x:v>
       </x:c>
       <x:c r="B20" s="10" t="str">
-        <x:v>A-10 §1, §4</x:v>
+        <x:v>Guía 10 sección 1, sección 4</x:v>
       </x:c>
       <x:c r="C20" s="10" t="str">
         <x:v>5 Movimiento</x:v>
@@ -3494,7 +3494,7 @@
         <x:v>RF-07</x:v>
       </x:c>
       <x:c r="B21" s="10" t="str">
-        <x:v>A-10 §1, RN-01</x:v>
+        <x:v>Guía 10 sección 1, RN-01</x:v>
       </x:c>
       <x:c r="C21" s="10" t="str">
         <x:v>5 Movimiento</x:v>
@@ -3514,7 +3514,7 @@
         <x:v>RF-08</x:v>
       </x:c>
       <x:c r="B22" s="10" t="str">
-        <x:v>A-10 §1, RN-04</x:v>
+        <x:v>Guía 10 sección 1, RN-04</x:v>
       </x:c>
       <x:c r="C22" s="10" t="str">
         <x:v>5 Movimiento</x:v>
@@ -3534,7 +3534,7 @@
         <x:v>RF-09</x:v>
       </x:c>
       <x:c r="B23" s="10" t="str">
-        <x:v>A-10 §1, RN-06; C-01 §3.3</x:v>
+        <x:v>Guía 10 sección 1, RN-06; caso sección 3.3</x:v>
       </x:c>
       <x:c r="C23" s="10" t="str">
         <x:v>2 Catálogo; 6 Alertas</x:v>
@@ -3554,7 +3554,7 @@
         <x:v>RF-10</x:v>
       </x:c>
       <x:c r="B24" s="10" t="str">
-        <x:v>A-10 §1; RD-03</x:v>
+        <x:v>Guía 10 sección 1; RD-03</x:v>
       </x:c>
       <x:c r="C24" s="10" t="str">
         <x:v>Transversal</x:v>

</xml_diff>

<commit_message>
feat: alta de producto con entrada inicial y ajuste por conteo físico
- Alta (RF-05): el producto nace con 0 unidades, como en SAP y Odoo; sus
  existencias entran con una Entrada. El Snackbar ofrece "Registrar
  entrada", que abre Movimiento con el producto y el tipo elegidos.
- Ajuste (RF-08, RN-04): se ingresa la cantidad contada (0 o más, distinta
  del disponible); la app muestra la diferencia y pide confirmar. Al
  confirmar, el stock pasa a lo contado y se guarda la diferencia con signo.
- Historial muestra el signo real de cada ajuste.
- Corrige el menú inferior: "Catálogo" restauraba Detalle y Movimiento en
  vez de volver al catálogo (saveState/restoreState).
- 45 pruebas unitarias (7 nuevas de alta y ajuste).
</commit_message>
<xml_diff>
--- a/docs/entregables/kaiju-requerimientos-guia-10.xlsx
+++ b/docs/entregables/kaiju-requerimientos-guia-10.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="Rcfdde051af7b4b5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Introducción y Contexto" sheetId="2" r:id="Re4c715eb11cd415a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Roles" sheetId="3" r:id="R6a49c86f5a5a4a06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Requerimientos (RF)" sheetId="4" r:id="R77dd051a2bf84926"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Reglas, RNF y RD" sheetId="5" r:id="Rc9cda29d58cc4705"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Alcance" sheetId="6" r:id="Rb2cf77a7def74b6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Pantallas" sheetId="7" r:id="R3a150acd58654b3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Modelo de Datos" sheetId="8" r:id="R709f3e2e1c2e4cf6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Trazabilidad" sheetId="9" r:id="R6b0148d014f84784"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 Checklist y Aceptación" sheetId="10" r:id="Rdaef51e4806b4ccc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="R2cac95139fe34a7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Introducción y Contexto" sheetId="2" r:id="Ra73f52cd9cca474c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Roles" sheetId="3" r:id="R31525bace67a4008"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Requerimientos (RF)" sheetId="4" r:id="R6298d405a6b543bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Reglas, RNF y RD" sheetId="5" r:id="R197603a205384f48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Alcance" sheetId="6" r:id="R46e2d1b0b8544fdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Pantallas" sheetId="7" r:id="R1ddf37e9bcf141b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Modelo de Datos" sheetId="8" r:id="R3f9694f0a4dd4a3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Trazabilidad" sheetId="9" r:id="Rd577b521bfa34cc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 Checklist y Aceptación" sheetId="10" r:id="R68e54f1f87014294"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1213,7 +1213,7 @@
         </x:is>
       </x:c>
       <x:c r="B13" s="10" t="str">
-        <x:v>App Android Kaiju: consultar existencias, registrar entradas y salidas con historial y detectar stock bajo. Implementa RF-01 a RF-10 de A-10, salvo el alta de producto (G10-02) y el cálculo del ajuste (G10-01). No integra sistemas externos ni usa datos reales. Detalle en hoja 5.</x:v>
+        <x:v>App Android Kaiju: consultar existencias, registrar entradas y salidas con historial y detectar stock bajo. Implementa RF-01 a RF-10 de Guía 10, salvo el alta de producto (G10-02) y el cálculo del ajuste (G10-01). No integra sistemas externos ni usa datos reales. Detalle en hoja 5.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="60" customHeight="1">
@@ -1223,7 +1223,7 @@
         </x:is>
       </x:c>
       <x:c r="B14" s="10" t="str">
-        <x:v>C-01 caso (CITT, 07-09-2026); N-04 plantilla; A-10 Guía 10 §1-9 y diagramas A-10-D1/D2; A-11 Guía 11 (recursos y permisos); guía extra del caso; Cuestionario IEEE 830. Sin acta de entrevista. Repositorio: docs/16 (auditoría) y docs/17 (prototipo).</x:v>
+        <x:v>Caso Kaiju (CITT, 07-09-2026); plantilla de requerimientos; Guía 10 (secciones 1 a 9) y sus diagramas de capas y navegación; Guía 11 (recursos y permisos); guía de persistencia con Room; guía extra del caso; Cuestionario IEEE 830. Sin acta de entrevista. Repositorio: docs/16 (auditoría) y docs/17 (prototipo).</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1251,7 +1251,7 @@
         <x:v>Producto</x:v>
       </x:c>
       <x:c r="B18" s="10" t="str">
-        <x:v>Definición documental provisional, no acordada: Artículo sobre el que se registran datos, cantidades y movimientos; C-01 §2.1/§3.2. Pendiente: Relación con materiales/insumos y atributos; P-06, P-07.</x:v>
+        <x:v>Definición documental provisional, no acordada: Artículo sobre el que se registran datos, cantidades y movimientos; caso sección 2.1/sección 3.2. Pendiente: Relación con materiales/insumos y atributos; P-06, P-07.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="60" customHeight="1">
@@ -1259,7 +1259,7 @@
         <x:v>Existencia / stock</x:v>
       </x:c>
       <x:c r="B19" s="10" t="str">
-        <x:v>Base A-10 §4-5: stockActual representa cantidad disponible; unidades reales y stock inicial al crear siguen pendientes G10-02. No acordado con cliente.</x:v>
+        <x:v>Base Guía 10 sección 4-5: stockActual representa cantidad disponible; unidades reales y stock inicial al crear siguen pendientes G10-02. No acordado con cliente.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="60" customHeight="1">
@@ -1267,7 +1267,7 @@
         <x:v>Movimiento</x:v>
       </x:c>
       <x:c r="B20" s="10" t="str">
-        <x:v>Base A-10 §4: ENTRADA, SALIDA_VENTA, SALIDA_CONSUMO y AJUSTE; guarda datos RN-05. Forma del ajuste pendiente G10-01. No acta comercial.</x:v>
+        <x:v>Base Guía 10 sección 4: ENTRADA, SALIDA_VENTA, SALIDA_CONSUMO y AJUSTE; guarda datos RN-05. Forma del ajuste pendiente G10-01. No acta comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="60" customHeight="1">
@@ -1275,7 +1275,7 @@
         <x:v>Venta</x:v>
       </x:c>
       <x:c r="B21" s="10" t="str">
-        <x:v>Base A-10 RF-07: salida por venta; no confirma documento comercial completo. C-01 menciona ventas. Composición adicional pendiente P-10.</x:v>
+        <x:v>Base Guía 10 RF-07: salida por venta; no confirma documento comercial completo. caso menciona ventas. Composición adicional pendiente P-10.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="60" customHeight="1">
@@ -1283,7 +1283,7 @@
         <x:v>Stock mínimo</x:v>
       </x:c>
       <x:c r="B22" s="10" t="str">
-        <x:v>Base A-10 RN-06: alerta si stockActual &lt;= stockMinimo. Umbral supuesto revisable del profesor; no validación comercial.</x:v>
+        <x:v>Base Guía 10 RN-06: alerta si stockActual &lt;= stockMinimo. Umbral supuesto revisable del profesor; no validación comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="60" customHeight="1">
@@ -1291,7 +1291,7 @@
         <x:v>Trazabilidad</x:v>
       </x:c>
       <x:c r="B23" s="10" t="str">
-        <x:v>Base A-10 RN-05: historial con fecha/tipo/cantidad/autor; no editar ni borrar movimientos, corregir mediante ajuste. Cliente aún sin validar.</x:v>
+        <x:v>Base Guía 10 RN-05: historial con fecha/tipo/cantidad/autor; no editar ni borrar movimientos, corregir mediante ajuste. Cliente aún sin validar.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1309,7 +1309,7 @@
         </x:is>
       </x:c>
       <x:c r="B26" s="10" t="str">
-        <x:v>Kaiju recibe, almacena, utiliza o vende productos, materiales e insumos. Hoy usa registros manuales y planillas que requieren actualización. C-01 §2.1-2.2.</x:v>
+        <x:v>Kaiju recibe, almacena, utiliza o vende productos, materiales e insumos. Hoy usa registros manuales y planillas que requieren actualización. caso sección 2.1-2.2.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="60" customHeight="1">
@@ -1319,7 +1319,7 @@
         </x:is>
       </x:c>
       <x:c r="B27" s="10" t="str">
-        <x:v>Posibles diferencias de existencias, movimientos omitidos y detección tardía de reposición dificultan el control y las decisiones. No hay mediciones aportadas. C-01 §2.3.</x:v>
+        <x:v>Posibles diferencias de existencias, movimientos omitidos y detección tardía de reposición dificultan el control y las decisiones. No hay mediciones aportadas. caso sección 2.3.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="60" customHeight="1">
@@ -1329,7 +1329,7 @@
         </x:is>
       </x:c>
       <x:c r="B28" s="10" t="str">
-        <x:v>Facilitar consulta y registro/revisión de movimientos para mejorar control y trazabilidad. Rapidez, actualización y mejora requieren criterios acordados. C-01 §2.4 y §4.1; P-11, P-15, P-18.</x:v>
+        <x:v>Facilitar consulta y registro/revisión de movimientos para mejorar control y trazabilidad. Rapidez, actualización y mejora requieren criterios acordados. caso sección 2.4 y sección 4.1; P-11, P-15, P-18.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="60" customHeight="1">
@@ -1339,7 +1339,7 @@
         </x:is>
       </x:c>
       <x:c r="B29" s="10" t="str">
-        <x:v>MVP Android académico. Integración con sistemas existentes no exigida; conexiones futuras deseables. RD académicas en hoja 4. C-01 §3.3-3.4 y §5.1.</x:v>
+        <x:v>MVP Android académico. Integración con sistemas existentes no exigida; conexiones futuras deseables. RD académicas en hoja 4. caso sección 3.3-3.4 y sección 5.1.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="60" customHeight="1">
@@ -1349,7 +1349,7 @@
         </x:is>
       </x:c>
       <x:c r="B30" s="10" t="str">
-        <x:v>Material académico autorizado: datos ficticios, sintéticos, agregados, públicos o anonimizados. Sin datos personales reales, registros productivos, accesos internos ni credenciales de Kaiju. C-01 §5.1; RD-05.</x:v>
+        <x:v>Material académico autorizado: datos ficticios, sintéticos, agregados, públicos o anonimizados. Sin datos personales reales, registros productivos, accesos internos ni credenciales de Kaiju. caso sección 5.1; RD-05.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="60" customHeight="1">
@@ -1359,7 +1359,7 @@
         </x:is>
       </x:c>
       <x:c r="B31" s="10" t="str">
-        <x:v>Sin acta: la entrevista aún no se agenda. Indicación docente (informada por Vicente el 14-10-2026): avanzar con el material entregado. RN-06 y permisos por perfil son supuestos revisables de A-10 §1. Decisiones técnicas reversibles en docs/17 §1; pendientes G10-01 a G10-10 en docs/11.</x:v>
+        <x:v>Sin acta: la entrevista aún no se agenda. Indicación docente (informada por Vicente el 14-10-2026): avanzar con el material entregado. RN-06 y permisos por perfil son supuestos revisables de Guía 10 sección 1. Decisiones técnicas reversibles en docs/17 sección 1; pendientes G10-01 a G10-10 en docs/11.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1431,7 +1431,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="10" t="str">
-        <x:v>ADMINISTRADOR en A-10 §4; perfil de prueba.</x:v>
+        <x:v>ADMINISTRADOR en Guía 10 sección 4; perfil de prueba.</x:v>
       </x:c>
       <x:c r="C5" s="10" t="str">
         <x:v>Consulta (RF-01 a RF-04); edita productos (RF-05; crear pendiente G10-02); registra entradas y ajustes (RF-06, RF-08); ve alertas (RF-09). No registra salidas: RF-07 no lo incluye (G10-04).</x:v>
@@ -1447,7 +1447,7 @@
         </x:is>
       </x:c>
       <x:c r="B6" s="10" t="str">
-        <x:v>VENDEDOR en A-10 §4; perfil de prueba.</x:v>
+        <x:v>VENDEDOR en Guía 10 sección 4; perfil de prueba.</x:v>
       </x:c>
       <x:c r="C6" s="10" t="str">
         <x:v>Consulta (RF-01 a RF-04) y registra salidas por venta (RF-07). Sin acceso a alertas, ajustes ni productos.</x:v>
@@ -1463,7 +1463,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>ENCARGADO_INVENTARIO en A-10 §4; perfil de prueba.</x:v>
+        <x:v>ENCARGADO_INVENTARIO en Guía 10 sección 4; perfil de prueba.</x:v>
       </x:c>
       <x:c r="C7" s="10" t="str">
         <x:v>Consulta (RF-01 a RF-04); registra entradas, salidas por venta o consumo y ajustes (RF-06 a RF-08); ve alertas y activa avisos (RF-09).</x:v>
@@ -1479,7 +1479,7 @@
         </x:is>
       </x:c>
       <x:c r="B8" s="10" t="str">
-        <x:v>Condicional en C-01; no es uno de los tres perfiles de la base A-10.</x:v>
+        <x:v>Condicional en caso; no es uno de los tres perfiles de la base Guía 10.</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
         <x:v>Consulta pública no incorporada automáticamente. Mantener P-05 y módulo propio pendiente.</x:v>
@@ -1595,10 +1595,10 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D6" s="10" t="str">
-        <x:v>A-10 §1-5, RF-01. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-01. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E6" s="10" t="str">
-        <x:v>Dado el login sin usuario elegido, cuando se toca Ingresar, entonces se muestra el error y no se ingresa. Dado un usuario elegido, cuando ingresa, entonces se ven su nombre y perfil y solo las acciones de su perfil (tabla A-10 §1).</x:v>
+        <x:v>Dado el login sin usuario elegido, cuando se toca Ingresar, entonces se muestra el error y no se ingresa. Dado un usuario elegido, cuando ingresa, entonces se ven su nombre y perfil y solo las acciones de su perfil (tabla Guía 10 sección 1).</x:v>
       </x:c>
       <x:c r="F6" s="10" t="str">
         <x:v>1 Login</x:v>
@@ -1617,7 +1617,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D7" s="10" t="str">
-        <x:v>A-10 §1-5, RF-02. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-02. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E7" s="10" t="str">
         <x:v>Dado el catálogo, cuando lo abre cualquier perfil, entonces cada producto muestra nombre, categoría, precio en CLP y cantidad disponible.</x:v>
@@ -1639,7 +1639,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D8" s="10" t="str">
-        <x:v>A-10 §1-5, RF-03. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-03. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E8" s="10" t="str">
         <x:v>Dado el catálogo, cuando se escribe parte del nombre o del código o se elige una categoría, entonces solo se listan los productos que cumplen ambos criterios. Semántica comercial pendiente G10-06.</x:v>
@@ -1661,7 +1661,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
-        <x:v>A-10 §1-5, RF-04. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-04. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E9" s="10" t="str">
         <x:v>Dado un producto con movimientos, cuando se abre su detalle, entonces se ven sus datos y su historial (fecha, tipo, cantidad, usuario, motivo) del más reciente al más antiguo.</x:v>
@@ -1693,10 +1693,10 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
-        <x:v>A-10 §1-5, RF-05. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-05. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
-        <x:v>Dado el administrador, cuando guarda con un campo inválido (A-10 §5), entonces el error aparece en ese campo y no se guarda. Cuando edita con datos válidos, entonces se guardan sin cambiar código ni stock. Alta: valida pero no guarda hasta resolver G10-02.</x:v>
+        <x:v>Dado el administrador, cuando guarda con un campo inválido (Guía 10 sección 5), entonces el error aparece en ese campo y no se guarda. Cuando edita con datos válidos, entonces se guardan sin cambiar código ni stock. Alta: valida pero no guarda hasta resolver G10-02.</x:v>
       </x:c>
       <x:c r="F11" s="10" t="str">
         <x:v>4 FormularioProducto</x:v>
@@ -1715,7 +1715,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D12" s="10" t="str">
-        <x:v>A-10 §1-5, RF-06. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-06. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E12" s="10" t="str">
         <x:v>Dado inventario o administrador, cuando registra una entrada con cantidad entera positiva, entonces el disponible aumenta en esa cantidad y el historial suma el movimiento con fecha y usuario, en la misma operación.</x:v>
@@ -1737,7 +1737,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D13" s="10" t="str">
-        <x:v>A-10 §1-5, RF-07. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-07. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E13" s="10" t="str">
         <x:v>Dado vendedor (venta) o inventario (venta o consumo), cuando registra una salida no mayor a lo disponible, entonces el disponible baja y queda el movimiento. Si la supera, se muestra el error y nada cambia (RN-01). Permiso del administrador pendiente G10-04.</x:v>
@@ -1759,7 +1759,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D14" s="10" t="str">
-        <x:v>A-10 §1-5, RF-08. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-08. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E14" s="10" t="str">
         <x:v>Dado inventario o administrador, cuando registra un ajuste sin motivo, entonces se muestra el error (RN-04). Efecto sobre el stock pendiente G10-01: con motivo, se informa el pendiente y no se registra.</x:v>
@@ -1791,7 +1791,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D16" s="10" t="str">
-        <x:v>A-10 §1-5, RF-09. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-09. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E16" s="10" t="str">
         <x:v>Dado un producto con disponible igual o menor a su mínimo, entonces aparece marcado en el catálogo y en Alertas (inventario y administrador), y al tocarlo se abre su detalle. Si un movimiento lo hace entrar en alerta y hay permiso, llega un aviso al teléfono.</x:v>
@@ -1813,7 +1813,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="D17" s="10" t="str">
-        <x:v>A-10 §1-5, RF-10. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
+        <x:v>Guía 10 sección 1-5, RF-10. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E17" s="10" t="str">
         <x:v>Dado un movimiento registrado, cuando se cierra la app y se vuelve a abrir, entonces productos e historial se conservan (Room). La sesión no se conserva: se vuelve a elegir usuario (G10-08).</x:v>
@@ -2016,7 +2016,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="F6" s="10" t="str">
-        <x:v>A-10 §1; §4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
+        <x:v>Guía 10 sección 1; sección 4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="100" customHeight="1">
@@ -2029,7 +2029,7 @@
         <x:v>Precio y mínimo</x:v>
       </x:c>
       <x:c r="C7" s="10" t="str">
-        <x:v>Precio &gt;0 y stock mínimo &gt;=0. A-10 §4-5 exige enteros, precio en CLP.</x:v>
+        <x:v>Precio &gt;0 y stock mínimo &gt;=0. Guía 10 sección 4-5 exige enteros, precio en CLP.</x:v>
       </x:c>
       <x:c r="D7" s="10" t="str">
         <x:v>Precio 1 y mínimo 0 cumplen; precio 0 o mínimo -1 no cumplen.</x:v>
@@ -2038,7 +2038,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="F7" s="10" t="str">
-        <x:v>A-10 §1; §4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
+        <x:v>Guía 10 sección 1; sección 4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="100" customHeight="1">
@@ -2060,7 +2060,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="F8" s="10" t="str">
-        <x:v>A-10 §1; §4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
+        <x:v>Guía 10 sección 1; sección 4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="100" customHeight="1">
@@ -2082,7 +2082,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="F9" s="10" t="str">
-        <x:v>A-10 §1; §4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
+        <x:v>Guía 10 sección 1; sección 4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="100" customHeight="1">
@@ -2104,7 +2104,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="F10" s="10" t="str">
-        <x:v>A-10 §1; §4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
+        <x:v>Guía 10 sección 1; sección 4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="100" customHeight="1">
@@ -2126,7 +2126,7 @@
         <x:v>Esencial</x:v>
       </x:c>
       <x:c r="F11" s="10" t="str">
-        <x:v>A-10 §1; §4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
+        <x:v>Guía 10 sección 1; sección 4-5 cuando corresponde. Base académica; no validación comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2188,7 +2188,7 @@
       </x:c>
       <x:c r="E15" s="10" t="n"/>
       <x:c r="F15" s="10" t="str">
-        <x:v>C-01 §4.1; RNF-01 candidato. Categoría y prioridad pendientes.</x:v>
+        <x:v>caso sección 4.1; RNF-01 candidato. Categoría y prioridad pendientes.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="100" customHeight="1">
@@ -2206,7 +2206,7 @@
       </x:c>
       <x:c r="E16" s="10" t="n"/>
       <x:c r="F16" s="10" t="str">
-        <x:v>C-01 §4.1 y §3.3; RNF-02 candidato. Categoría y prioridad pendientes.</x:v>
+        <x:v>caso sección 4.1 y sección 3.3; RNF-02 candidato. Categoría y prioridad pendientes.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="100" customHeight="1">
@@ -2224,7 +2224,7 @@
       </x:c>
       <x:c r="E17" s="10" t="n"/>
       <x:c r="F17" s="10" t="str">
-        <x:v>C-01 §3.3; RNF-03 candidato. Categoría y prioridad pendientes.</x:v>
+        <x:v>caso sección 3.3; RNF-03 candidato. Categoría y prioridad pendientes.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
@@ -2539,7 +2539,7 @@
         <x:v>Sesión y consulta</x:v>
       </x:c>
       <x:c r="B6" s="10" t="str">
-        <x:v>RF-01 a RF-04: explícitos A-10; no autenticación productiva.</x:v>
+        <x:v>RF-01 a RF-04: explícitos Guía 10; no autenticación productiva.</x:v>
       </x:c>
       <x:c r="C6" s="10" t="str">
         <x:v>RF-01 a RF-04</x:v>
@@ -2550,7 +2550,7 @@
         <x:v>Crear y editar productos</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>Editar implementado (A-10 RF-05). Crear valida, pero no guarda hasta resolver G10-02; código no editable (G10-03).</x:v>
+        <x:v>Editar implementado (Guía 10 RF-05). Crear valida, pero no guarda hasta resolver G10-02; código no editable (G10-03).</x:v>
       </x:c>
       <x:c r="C7" s="10" t="str">
         <x:v>RF-05</x:v>
@@ -2561,7 +2561,7 @@
         <x:v>Entradas, salidas y ajustes</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
-        <x:v>Entradas y salidas implementadas (A-10 RF-06/07). Ajuste valida el motivo; su efecto espera G10-01.</x:v>
+        <x:v>Entradas y salidas implementadas (Guía 10 RF-06/07). Ajuste valida el motivo; su efecto espera G10-01.</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
         <x:v>RF-06 a RF-08</x:v>
@@ -2572,7 +2572,7 @@
         <x:v>Alertas, marca de stock bajo y aviso del teléfono</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>A-10 RN-06 y RF-09; aviso por notificación según C-01 §3.3 y RD-04. Umbral revisable.</x:v>
+        <x:v>Guía 10 RN-06 y RF-09; aviso por notificación según caso sección 3.3 y RD-04. Umbral revisable.</x:v>
       </x:c>
       <x:c r="C9" s="10" t="str">
         <x:v>RF-09</x:v>
@@ -2594,7 +2594,7 @@
         <x:v>Lector de códigos para elegir el producto</x:v>
       </x:c>
       <x:c r="B11" s="10" t="str">
-        <x:v>C-01 §3.3 menciona la cámara para leer códigos; cumple RD-04 junto con las notificaciones. Sin permiso de cámara.</x:v>
+        <x:v>caso sección 3.3 menciona la cámara para leer códigos; cumple RD-04 junto con las notificaciones. Sin permiso de cámara.</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
         <x:v>RF-06, RF-07</x:v>
@@ -2637,7 +2637,7 @@
         <x:v>Integración con sistemas de venta, catálogos digitales o facturación</x:v>
       </x:c>
       <x:c r="B15" s="10" t="str">
-        <x:v>C-01 §3.4 y §5.1: no se exige para el MVP; se considera deseable a futuro.</x:v>
+        <x:v>caso sección 3.4 y sección 5.1: no se exige para el MVP; se considera deseable a futuro.</x:v>
       </x:c>
       <x:c r="C15" s="10" t="str">
         <x:v>Sí</x:v>
@@ -2648,7 +2648,7 @@
         <x:v>Uso de datos reales, credenciales o accesos de Kaiju</x:v>
       </x:c>
       <x:c r="B16" s="10" t="str">
-        <x:v>Prohibido por C-01 §5.1 y RD-05: solo datos ficticios.</x:v>
+        <x:v>Prohibido por caso sección 5.1 y RD-05: solo datos ficticios.</x:v>
       </x:c>
       <x:c r="C16" s="10" t="str">
         <x:v>No</x:v>
@@ -2720,7 +2720,7 @@
         <x:v>Navegación y permisos</x:v>
       </x:c>
       <x:c r="B24" s="10" t="str">
-        <x:v>Destinos resueltos A-10-D2; variación por rol y algunas salidas pendientes G10-04.</x:v>
+        <x:v>Destinos resueltos diagrama 2 de la Guía 10; variación por rol y algunas salidas pendientes G10-04.</x:v>
       </x:c>
       <x:c r="C24" s="10" t="str">
         <x:v>Docente / cliente según validación.</x:v>
@@ -2762,7 +2762,7 @@
         <x:v>Equipo, evaluación y módulo propio</x:v>
       </x:c>
       <x:c r="B27" s="10" t="str">
-        <x:v>Aceptación del trabajo individual y evidencia sin Trello (IE 2.3.2). Módulo propio: más/menos vendidos o tendencias (C-01 §4.1) requieren medida y período (P-13, P-14).</x:v>
+        <x:v>Aceptación del trabajo individual y evidencia sin Trello (IE 2.3.2). Módulo propio: más/menos vendidos o tendencias (caso sección 4.1) requieren medida y período (P-13, P-14).</x:v>
       </x:c>
       <x:c r="C27" s="10" t="str">
         <x:v>Docente (evaluación); cliente (módulo).</x:v>
@@ -2851,19 +2851,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B5" s="10" t="str">
-        <x:v>PantallaLogin (A-10 §2; A-10-D2).</x:v>
+        <x:v>PantallaLogin (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="C5" s="10" t="str">
-        <x:v>Tres usuarios de prueba (A-10 §2; A-10-D2).</x:v>
+        <x:v>Tres usuarios de prueba (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="D5" s="10" t="str">
-        <x:v>Entrada de app (A-10 §2; A-10-D2).</x:v>
+        <x:v>Entrada de app (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="E5" s="10" t="str">
-        <x:v>Elegir usuario obligatorio, error desde SesionViewModel. (A-10 §2; A-10-D2).</x:v>
+        <x:v>Elegir usuario obligatorio, error desde SesionViewModel. (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="F5" s="10" t="str">
-        <x:v>RF-01 (A-10 §2; A-10-D2).</x:v>
+        <x:v>RF-01 (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="100" customHeight="1">
@@ -2871,19 +2871,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B6" s="10" t="str">
-        <x:v>PantallaCatalogo (A-10 §2; A-10-D2).</x:v>
+        <x:v>PantallaCatalogo (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="C6" s="10" t="str">
-        <x:v>Tres perfiles base (A-10 §2; A-10-D2).</x:v>
+        <x:v>Tres perfiles base (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="D6" s="10" t="str">
-        <x:v>Login; menú inferior (A-10 §2; A-10-D2).</x:v>
+        <x:v>Login; menú inferior (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="E6" s="10" t="str">
-        <x:v>Nombre/categoría/precio/cantidad, búsqueda/filtro, marca bajo mínimo. (A-10 §2; A-10-D2).</x:v>
+        <x:v>Nombre/categoría/precio/cantidad, búsqueda/filtro, marca bajo mínimo. (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="F6" s="10" t="str">
-        <x:v>RF-02/03/09 (A-10 §2; A-10-D2).</x:v>
+        <x:v>RF-02/03/09 (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="100" customHeight="1">
@@ -2891,19 +2891,19 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>PantallaDetalleProducto (A-10 §2; A-10-D2).</x:v>
+        <x:v>PantallaDetalleProducto (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="C7" s="10" t="str">
-        <x:v>Tres perfiles base (A-10 §2; A-10-D2).</x:v>
+        <x:v>Tres perfiles base (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="D7" s="10" t="str">
-        <x:v>Catálogo al tocar producto; alerta al tocarla (A-10 §2; A-10-D2).</x:v>
+        <x:v>Catálogo al tocar producto; alerta al tocarla (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="E7" s="10" t="str">
-        <x:v>Datos e historial por producto, recientes primero. (A-10 §2; A-10-D2).</x:v>
+        <x:v>Datos e historial por producto, recientes primero. (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="F7" s="10" t="str">
-        <x:v>RF-04 (A-10 §2; A-10-D2).</x:v>
+        <x:v>RF-04 (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="100" customHeight="1">
@@ -2911,19 +2911,19 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
-        <x:v>PantallaFormularioProducto (A-10 §2; A-10-D2).</x:v>
+        <x:v>PantallaFormularioProducto (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
-        <x:v>Administrador (A-10 §2; A-10-D2).</x:v>
+        <x:v>Administrador (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="D8" s="10" t="str">
-        <x:v>Botón + del Catálogo (crear) y botón Editar en el detalle (A-10 §2; A-10-D2).</x:v>
+        <x:v>Botón + del Catálogo (crear) y botón Editar en el detalle (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="E8" s="10" t="str">
-        <x:v>Validaciones §5. Stock inicial/código editable pendientes G10-02/03. (A-10 §2; A-10-D2).</x:v>
+        <x:v>Validaciones sección 5. Stock inicial/código editable pendientes G10-02/03. (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="F8" s="10" t="str">
-        <x:v>RF-05 (A-10 §2; A-10-D2).</x:v>
+        <x:v>RF-05 (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="100" customHeight="1">
@@ -2931,19 +2931,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>PantallaMovimiento (A-10 §2; A-10-D2).</x:v>
+        <x:v>PantallaMovimiento (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="C9" s="10" t="str">
-        <x:v>Según perfil y tipo; permisos G10-04 (A-10 §2; A-10-D2).</x:v>
+        <x:v>Según perfil y tipo; permisos G10-04 (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
-        <x:v>Menú inferior; registrar desde detalle (A-10 §2; A-10-D2).</x:v>
+        <x:v>Menú inferior; registrar desde detalle (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="E9" s="10" t="str">
-        <x:v>Producto (lista o lector de códigos), tipo según perfil, cantidad entera positiva, motivo obligatorio en ajuste. Fórmula del ajuste pendiente G10-01. (A-10 §2, §5)</x:v>
+        <x:v>Producto (lista o lector de códigos), tipo según perfil, cantidad entera positiva, motivo obligatorio en ajuste. Fórmula del ajuste pendiente G10-01. (Guía 10 sección 2, sección 5)</x:v>
       </x:c>
       <x:c r="F9" s="10" t="str">
-        <x:v>RF-06/07/08 (A-10 §2; A-10-D2).</x:v>
+        <x:v>RF-06/07/08 (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="100" customHeight="1">
@@ -2951,19 +2951,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B10" s="10" t="str">
-        <x:v>PantallaAlertas (A-10 §2; A-10-D2).</x:v>
+        <x:v>PantallaAlertas (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="C10" s="10" t="str">
-        <x:v>Inventario y administrador (A-10 §2; A-10-D2).</x:v>
+        <x:v>Inventario y administrador (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="D10" s="10" t="str">
-        <x:v>Menú inferior; variación por perfil por precisar (A-10 §2; A-10-D2).</x:v>
+        <x:v>Menú inferior; variación por perfil por precisar (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="E10" s="10" t="str">
-        <x:v>Lista bajo mínimo; tocar abre detalle. Tarjeta para activar avisos con permiso POST_NOTIFICATIONS (A-11 §4). (A-10 §2)</x:v>
+        <x:v>Lista bajo mínimo; tocar abre detalle. Tarjeta para activar avisos con permiso POST_NOTIFICATIONS (Guía 11 sección 4). (Guía 10 sección 2)</x:v>
       </x:c>
       <x:c r="F10" s="10" t="str">
-        <x:v>RF-09 (A-10 §2; A-10-D2).</x:v>
+        <x:v>RF-09 (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
@@ -3069,13 +3069,13 @@
         <x:v>Producto</x:v>
       </x:c>
       <x:c r="B5" s="10" t="str">
-        <x:v>codigo, nombre, descripcion, categoria, tipo, precio Int CLP, stockActual, stockMinimo, detalle opcional texto. Otros tipos pendientes. A-10 §4.</x:v>
+        <x:v>codigo, nombre, descripcion, categoria, tipo, precio Int CLP, stockActual, stockMinimo, detalle opcional texto. Otros tipos pendientes. Guía 10 sección 4.</x:v>
       </x:c>
       <x:c r="C5" s="10" t="str">
         <x:v>Room</x:v>
       </x:c>
       <x:c r="D5" s="10" t="str">
-        <x:v>Clave primaria: codigo. Un producto tiene muchos movimientos. stockActual solo cambia al registrar un movimiento (A-10 §4).</x:v>
+        <x:v>Clave primaria: codigo. Un producto tiene muchos movimientos. stockActual solo cambia al registrar un movimiento (Guía 10 sección 4).</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="75" customHeight="1">
@@ -3083,7 +3083,7 @@
         <x:v>Movimiento</x:v>
       </x:c>
       <x:c r="B6" s="10" t="str">
-        <x:v>id, codigoProducto, tipo (enum), cantidad, motivo, fecha, usuario. Tipos/políticas pendientes G10-07. A-10 §4.</x:v>
+        <x:v>id, codigoProducto, tipo (enum), cantidad, motivo, fecha, usuario. Tipos/políticas pendientes G10-07. Guía 10 sección 4.</x:v>
       </x:c>
       <x:c r="C6" s="10" t="str">
         <x:v>Room</x:v>
@@ -3097,7 +3097,7 @@
         <x:v>Usuario</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>id, nombre, rol (enum). Tres usuarios ficticios; no personas reales. A-10 §4.</x:v>
+        <x:v>id, nombre, rol (enum). Tres usuarios ficticios; no personas reales. Guía 10 sección 4.</x:v>
       </x:c>
       <x:c r="C7" s="10" t="n"/>
       <x:c r="D7" s="10" t="str">
@@ -3109,11 +3109,11 @@
         <x:v>Enums</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
-        <x:v>TipoMovimiento: ENTRADA, SALIDA_VENTA, SALIDA_CONSUMO, AJUSTE. Rol: ADMINISTRADOR, VENDEDOR, ENCARGADO_INVENTARIO. A-10 §4.</x:v>
+        <x:v>TipoMovimiento: ENTRADA, SALIDA_VENTA, SALIDA_CONSUMO, AJUSTE. Rol: ADMINISTRADOR, VENDEDOR, ENCARGADO_INVENTARIO. Guía 10 sección 4.</x:v>
       </x:c>
       <x:c r="C8" s="10" t="n"/>
       <x:c r="D8" s="10" t="str">
-        <x:v>A-10 §4. No son tablas obligatorias independientes. Memoria ahora; persistencia por decidir después.</x:v>
+        <x:v>Guía 10 sección 4. No son tablas obligatorias independientes. Memoria ahora; persistencia por decidir después.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
@@ -3318,7 +3318,7 @@
         </x:is>
       </x:c>
       <x:c r="B11" s="10" t="str">
-        <x:v>Interna: RF-02 y RF-03. Público general condicional (C-01 §3.1), no incluido; pendiente P-05.</x:v>
+        <x:v>Interna: RF-02 y RF-03. Público general condicional (caso sección 3.1), no incluido; pendiente P-05.</x:v>
       </x:c>
       <x:c r="C11" s="12" t="n"/>
       <x:c r="D11" s="12" t="n"/>
@@ -3374,7 +3374,7 @@
         <x:v>RF-01</x:v>
       </x:c>
       <x:c r="B15" s="10" t="str">
-        <x:v>A-10 §1</x:v>
+        <x:v>Guía 10 sección 1</x:v>
       </x:c>
       <x:c r="C15" s="10" t="str">
         <x:v>1 Login</x:v>
@@ -3394,7 +3394,7 @@
         <x:v>RF-02</x:v>
       </x:c>
       <x:c r="B16" s="10" t="str">
-        <x:v>A-10 §1</x:v>
+        <x:v>Guía 10 sección 1</x:v>
       </x:c>
       <x:c r="C16" s="10" t="str">
         <x:v>2 Catálogo</x:v>
@@ -3414,7 +3414,7 @@
         <x:v>RF-03</x:v>
       </x:c>
       <x:c r="B17" s="10" t="str">
-        <x:v>A-10 §1</x:v>
+        <x:v>Guía 10 sección 1</x:v>
       </x:c>
       <x:c r="C17" s="10" t="str">
         <x:v>2 Catálogo</x:v>
@@ -3434,7 +3434,7 @@
         <x:v>RF-04</x:v>
       </x:c>
       <x:c r="B18" s="10" t="str">
-        <x:v>A-10 §1-2</x:v>
+        <x:v>Guía 10 sección 1-2</x:v>
       </x:c>
       <x:c r="C18" s="10" t="str">
         <x:v>3 Detalle</x:v>
@@ -3454,7 +3454,7 @@
         <x:v>RF-05</x:v>
       </x:c>
       <x:c r="B19" s="10" t="str">
-        <x:v>A-10 §1, §5</x:v>
+        <x:v>Guía 10 sección 1, sección 5</x:v>
       </x:c>
       <x:c r="C19" s="10" t="str">
         <x:v>4 Formulario producto</x:v>
@@ -3474,7 +3474,7 @@
         <x:v>RF-06</x:v>
       </x:c>
       <x:c r="B20" s="10" t="str">
-        <x:v>A-10 §1, §4</x:v>
+        <x:v>Guía 10 sección 1, sección 4</x:v>
       </x:c>
       <x:c r="C20" s="10" t="str">
         <x:v>5 Movimiento</x:v>
@@ -3494,7 +3494,7 @@
         <x:v>RF-07</x:v>
       </x:c>
       <x:c r="B21" s="10" t="str">
-        <x:v>A-10 §1, RN-01</x:v>
+        <x:v>Guía 10 sección 1, RN-01</x:v>
       </x:c>
       <x:c r="C21" s="10" t="str">
         <x:v>5 Movimiento</x:v>
@@ -3514,7 +3514,7 @@
         <x:v>RF-08</x:v>
       </x:c>
       <x:c r="B22" s="10" t="str">
-        <x:v>A-10 §1, RN-04</x:v>
+        <x:v>Guía 10 sección 1, RN-04</x:v>
       </x:c>
       <x:c r="C22" s="10" t="str">
         <x:v>5 Movimiento</x:v>
@@ -3534,7 +3534,7 @@
         <x:v>RF-09</x:v>
       </x:c>
       <x:c r="B23" s="10" t="str">
-        <x:v>A-10 §1, RN-06; C-01 §3.3</x:v>
+        <x:v>Guía 10 sección 1, RN-06; caso sección 3.3</x:v>
       </x:c>
       <x:c r="C23" s="10" t="str">
         <x:v>2 Catálogo; 6 Alertas</x:v>
@@ -3554,7 +3554,7 @@
         <x:v>RF-10</x:v>
       </x:c>
       <x:c r="B24" s="10" t="str">
-        <x:v>A-10 §1; RD-03</x:v>
+        <x:v>Guía 10 sección 1; RD-03</x:v>
       </x:c>
       <x:c r="C24" s="10" t="str">
         <x:v>Transversal</x:v>

</xml_diff>

<commit_message>
docs: evidencia final y contraste con la rúbrica del encargo
- 29 capturas del emulador (API 36) con índice por requisito:
  formularios, movimientos, ajuste, permisos, notificación real,
  perfiles, persistencia tras cerrar el proceso y rotación.
- docs/19: requisito por requisito de las Reglas de Entrega, la
  rúbrica del Encargo, la Guía 10 (B-01 a B-09), la Guía 11 y la
  Guía de Room, con su código, prueba y captura.
- Reglas de Entrega guardadas como fuente (A-REGLAS).
- Word de evidencia final con las capturas; README, bitácora,
  evidencia del código, tablero y plantilla de requerimientos al día
  (stock inicial y ajuste como decisiones revisables, 45 pruebas
  unitarias y 3 de Room aprobadas en el emulador).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/entregables/kaiju-requerimientos-guia-10.xlsx
+++ b/docs/entregables/kaiju-requerimientos-guia-10.xlsx
@@ -904,7 +904,9 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
-      <x:c r="A6" s="10" t="n"/>
+      <x:c r="A6" s="10" t="str">
+        <x:v>X</x:v>
+      </x:c>
       <x:c r="B6" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Proyecto creado con estructura MVVM (ui, viewmodel, model) y dependencias (Compose, Material 3, Navigation, Room, DataStore).</x:t>
@@ -963,7 +965,7 @@
         </x:is>
       </x:c>
       <x:c r="C10" s="10" t="str">
-        <x:v>Login, producto y movimiento; 40 pruebas unitarias.</x:v>
+        <x:v>Login, producto y movimiento; 45 pruebas unitarias.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -980,47 +982,55 @@
       </x:c>
     </x:row>
     <x:row r="12" ht="48" customHeight="1">
-      <x:c r="A12" s="10" t="n"/>
+      <x:c r="A12" s="10" t="str">
+        <x:v>X</x:v>
+      </x:c>
       <x:c r="B12" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Persistencia local funcionando (Room y/o DataStore).</x:t>
         </x:is>
       </x:c>
       <x:c r="C12" s="10" t="str">
-        <x:v>Implementado con Room; falta comprobar en teléfono (InventarioDaoTest y pauta paso 19).</x:v>
+        <x:v>Room funcionando: 3/3 pruebas en el emulador y captura 26 (datos tras cerrar el proceso).</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
-      <x:c r="A13" s="10" t="n"/>
+      <x:c r="A13" s="10" t="str">
+        <x:v>X</x:v>
+      </x:c>
       <x:c r="B13" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Dos recursos nativos integrados y funcionando sin capturar datos reales de personas.</x:t>
         </x:is>
       </x:c>
       <x:c r="C13" s="10" t="str">
-        <x:v>Notificaciones y lector de códigos implementados; falta probar en teléfono.</x:v>
+        <x:v>Notificaciones con permiso (capturas 18 a 23) y lector de códigos (en el emulador muestra la alternativa, captura 16).</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
-      <x:c r="A14" s="10" t="n"/>
+      <x:c r="A14" s="10" t="str">
+        <x:v>X</x:v>
+      </x:c>
       <x:c r="B14" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Animaciones que aporten fluidez.</x:t>
         </x:is>
       </x:c>
       <x:c r="C14" s="10" t="str">
-        <x:v>Implementadas; falta revisión visual.</x:v>
+        <x:v>Cinco animaciones con propósito (README y docs/19), revisadas en el emulador.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
-      <x:c r="A15" s="10" t="n"/>
+      <x:c r="A15" s="10" t="str">
+        <x:v>X</x:v>
+      </x:c>
       <x:c r="B15" s="8" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Repositorio GitHub con commits de todos los integrantes y tablero Trello al día.</x:t>
         </x:is>
       </x:c>
       <x:c r="C15" s="10" t="str">
-        <x:v>Commits de un solo integrante (trabajo individual). Sin Trello: consultar al docente.</x:v>
+        <x:v>Commits de un solo integrante (trabajo individual). Trello al día desde el 14-10-2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1213,7 +1223,7 @@
         </x:is>
       </x:c>
       <x:c r="B13" s="10" t="str">
-        <x:v>App Android Kaiju: consultar existencias, registrar entradas y salidas con historial y detectar stock bajo. Implementa RF-01 a RF-10 de Guía 10, salvo el alta de producto (G10-02) y el cálculo del ajuste (G10-01). No integra sistemas externos ni usa datos reales. Detalle en hoja 5.</x:v>
+        <x:v>App Android Kaiju: consultar existencias, registrar entradas y salidas con historial y detectar stock bajo. Implementa RF-01 a RF-10 de Guía 10. El stock inicial del alta (G10-02) y el cálculo del ajuste (G10-01) se resolvieron como decisión técnica revisable, docs/18; no son acuerdo del cliente. No integra sistemas externos ni usa datos reales. Detalle en hoja 5.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="60" customHeight="1">
@@ -1259,7 +1269,7 @@
         <x:v>Existencia / stock</x:v>
       </x:c>
       <x:c r="B19" s="10" t="str">
-        <x:v>Base Guía 10 sección 4-5: stockActual representa cantidad disponible; unidades reales y stock inicial al crear siguen pendientes G10-02. No acordado con cliente.</x:v>
+        <x:v>Base Guía 10 sección 4-5: stockActual representa la cantidad disponible. Un producto nuevo parte en 0 y su stock entra con una Entrada (G10-02, decisión técnica revisable, docs/18). Unidades reales no acordadas con el cliente.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="60" customHeight="1">
@@ -1267,7 +1277,7 @@
         <x:v>Movimiento</x:v>
       </x:c>
       <x:c r="B20" s="10" t="str">
-        <x:v>Base Guía 10 sección 4: ENTRADA, SALIDA_VENTA, SALIDA_CONSUMO y AJUSTE; guarda datos RN-05. Forma del ajuste pendiente G10-01. No acta comercial.</x:v>
+        <x:v>Base Guía 10 sección 4: ENTRADA, SALIDA_VENTA, SALIDA_CONSUMO y AJUSTE; guarda los datos de RN-05. El ajuste es un conteo físico que guarda la diferencia (G10-01, decisión técnica revisable, docs/18). No es acta comercial.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="60" customHeight="1">
@@ -1434,7 +1444,7 @@
         <x:v>ADMINISTRADOR en Guía 10 sección 4; perfil de prueba.</x:v>
       </x:c>
       <x:c r="C5" s="10" t="str">
-        <x:v>Consulta (RF-01 a RF-04); edita productos (RF-05; crear pendiente G10-02); registra entradas y ajustes (RF-06, RF-08); ve alertas (RF-09). No registra salidas: RF-07 no lo incluye (G10-04).</x:v>
+        <x:v>Consulta (RF-01 a RF-04); crea y edita productos (RF-05); registra entradas y ajustes (RF-06, RF-08); ve alertas (RF-09). No registra salidas: RF-07 no lo incluye (G10-04).</x:v>
       </x:c>
       <x:c r="D5" s="10" t="str">
         <x:v>Nivel técnico y frecuencia sin información; preguntar P-23.</x:v>
@@ -1696,7 +1706,7 @@
         <x:v>Guía 10 sección 1-5, RF-05. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E11" s="10" t="str">
-        <x:v>Dado el administrador, cuando guarda con un campo inválido (Guía 10 sección 5), entonces el error aparece en ese campo y no se guarda. Cuando edita con datos válidos, entonces se guardan sin cambiar código ni stock. Alta: valida pero no guarda hasta resolver G10-02.</x:v>
+        <x:v>Dado el administrador, cuando guarda con un campo inválido (Guía 10 sección 5), entonces el error aparece en ese campo y no se guarda. Cuando crea con datos válidos, el producto aparece en el catálogo con 0 unidades y se ofrece registrar su entrada (G10-02, decisión técnica revisable, docs/18). Cuando edita con datos válidos, se guardan sin cambiar código ni stock.</x:v>
       </x:c>
       <x:c r="F11" s="10" t="str">
         <x:v>4 FormularioProducto</x:v>
@@ -1762,7 +1772,7 @@
         <x:v>Guía 10 sección 1-5, RF-08. Base académica, no acta cliente; prioridad esencial para base docente.</x:v>
       </x:c>
       <x:c r="E14" s="10" t="str">
-        <x:v>Dado inventario o administrador, cuando registra un ajuste sin motivo, entonces se muestra el error (RN-04). Efecto sobre el stock pendiente G10-01: con motivo, se informa el pendiente y no se registra.</x:v>
+        <x:v>Dado inventario o administrador, cuando registra un ajuste sin motivo, entonces se muestra el error (RN-04). Con motivo, se ingresa la cantidad contada (distinta de lo disponible), se confirma la diferencia y el disponible pasa a ser lo contado; el movimiento guarda la diferencia con signo (G10-01, decisión técnica revisable, docs/18).</x:v>
       </x:c>
       <x:c r="F14" s="10" t="str">
         <x:v>5 Movimiento</x:v>
@@ -2076,7 +2086,7 @@
         <x:v>Todo ajuste exige motivo. No define fórmula del ajuste ni obliga motivo en otros tipos.</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
-        <x:v>Ajuste sin motivo no cumple; con motivo satisface esta regla, sujeto a aclarar G10-01.</x:v>
+        <x:v>Un ajuste sin motivo no cumple; con motivo satisface esta regla. El cálculo como conteo físico es decisión técnica revisable, docs/18 (G10-01).</x:v>
       </x:c>
       <x:c r="E9" s="10" t="str">
         <x:v>Esencial</x:v>
@@ -2098,7 +2108,7 @@
         <x:v>Cada movimiento conserva fecha, tipo, cantidad y autor; no editar/borrar; corregir mediante ajuste.</x:v>
       </x:c>
       <x:c r="D10" s="10" t="str">
-        <x:v>Registro conserva los cuatro datos; no hay edición/borrado del movimiento. Fórmula de corrección pendiente G10-01.</x:v>
+        <x:v>El registro conserva los cuatro datos; no hay edición ni borrado del movimiento. Un error se corrige con un ajuste por conteo (G10-01, decisión técnica revisable, docs/18).</x:v>
       </x:c>
       <x:c r="E10" s="10" t="str">
         <x:v>Esencial</x:v>
@@ -2550,7 +2560,7 @@
         <x:v>Crear y editar productos</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>Editar implementado (Guía 10 RF-05). Crear valida, pero no guarda hasta resolver G10-02; código no editable (G10-03).</x:v>
+        <x:v>Crear y editar implementados (Guía 10 RF-05). El producto nuevo parte en 0 y se ofrece registrar su entrada (G10-02, decisión técnica revisable, docs/18); el código no es editable (G10-03).</x:v>
       </x:c>
       <x:c r="C7" s="10" t="str">
         <x:v>RF-05</x:v>
@@ -2561,7 +2571,7 @@
         <x:v>Entradas, salidas y ajustes</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
-        <x:v>Entradas y salidas implementadas (Guía 10 RF-06/07). Ajuste valida el motivo; su efecto espera G10-01.</x:v>
+        <x:v>Entradas, salidas y ajuste implementados (Guía 10 RF-06/07/08). El ajuste es un conteo físico con confirmación (G10-01, decisión técnica revisable, docs/18).</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
         <x:v>RF-06 a RF-08</x:v>
@@ -2706,7 +2716,7 @@
         <x:v>Stock inicial, ajuste y código</x:v>
       </x:c>
       <x:c r="B23" s="10" t="str">
-        <x:v>G10-01/02/03: efecto de ajuste, alta y relación historial.</x:v>
+        <x:v>G10-01 y G10-02 resueltos como decisión técnica revisable (docs/18); confirmar con el docente y el cliente. G10-03: relación del código con el historial.</x:v>
       </x:c>
       <x:c r="C23" s="10" t="str">
         <x:v>Docente; contraste comercial si corresponde.</x:v>
@@ -2762,7 +2772,7 @@
         <x:v>Equipo, evaluación y módulo propio</x:v>
       </x:c>
       <x:c r="B27" s="10" t="str">
-        <x:v>Aceptación del trabajo individual y evidencia sin Trello (IE 2.3.2). Módulo propio: más/menos vendidos o tendencias (caso sección 4.1) requieren medida y período (P-13, P-14).</x:v>
+        <x:v>Aceptación del trabajo individual (IE 2.3.2). Módulo propio: más/menos vendidos o tendencias (caso sección 4.1) requieren medida y período (P-13, P-14).</x:v>
       </x:c>
       <x:c r="C27" s="10" t="str">
         <x:v>Docente (evaluación); cliente (módulo).</x:v>
@@ -2920,7 +2930,7 @@
         <x:v>Botón + del Catálogo (crear) y botón Editar en el detalle (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="E8" s="10" t="str">
-        <x:v>Validaciones sección 5. Stock inicial/código editable pendientes G10-02/03. (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
+        <x:v>Validaciones sección 5. El producto nuevo parte en 0 (G10-02, decisión técnica revisable, docs/18); el código no es editable (G10-03). (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="F8" s="10" t="str">
         <x:v>RF-05 (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
@@ -2940,7 +2950,7 @@
         <x:v>Menú inferior; registrar desde detalle (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
       </x:c>
       <x:c r="E9" s="10" t="str">
-        <x:v>Producto (lista o lector de códigos), tipo según perfil, cantidad entera positiva, motivo obligatorio en ajuste. Fórmula del ajuste pendiente G10-01. (Guía 10 sección 2, sección 5)</x:v>
+        <x:v>Producto (lista o lector de códigos), tipo según perfil, cantidad entera positiva, motivo obligatorio en ajuste. Ajuste como conteo con confirmación (G10-01, decisión técnica revisable, docs/18). (Guía 10 sección 2, sección 5)</x:v>
       </x:c>
       <x:c r="F9" s="10" t="str">
         <x:v>RF-06/07/08 (Guía 10 sección 2; diagrama 2 de la Guía 10).</x:v>
@@ -3113,7 +3123,7 @@
       </x:c>
       <x:c r="C8" s="10" t="n"/>
       <x:c r="D8" s="10" t="str">
-        <x:v>Guía 10 sección 4. No son tablas obligatorias independientes. Memoria ahora; persistencia por decidir después.</x:v>
+        <x:v>Guía 10 sección 4. Se guardan con Room en dos tablas (productos y movimientos); el Usuario va dentro de cada movimiento.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
@@ -3262,7 +3272,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>RF-09 y RN-06 (alertas y aviso), RN-01 (sin stock negativo), RF-08 ajuste con motivo (efecto pendiente G10-01). Sin métrica acordada para medir la disminución (P-18).</x:v>
+        <x:v>RF-09 y RN-06 (alertas y aviso), RN-01 (sin stock negativo), RF-08 ajuste por conteo con motivo (G10-01, decisión revisable). Sin métrica acordada para medir la disminución (P-18).</x:v>
       </x:c>
       <x:c r="C7" s="12" t="n"/>
       <x:c r="D7" s="12" t="n"/>
@@ -3483,7 +3493,7 @@
         <x:v>InventarioViewModel.registrarMovimiento; InventarioDao</x:v>
       </x:c>
       <x:c r="E20" s="10" t="str">
-        <x:v>entradaSumaStock...; InventarioDaoTest (en teléfono)</x:v>
+        <x:v>entradaSumaStock...; InventarioDaoTest (3/3 en emulador, 15-10-2026)</x:v>
       </x:c>
       <x:c r="F20" s="10" t="str">
         <x:v>IE 2.1.2, IE 2.2.1, IE 2.3.1</x:v>
@@ -3563,7 +3573,7 @@
         <x:v>database/BaseDeDatosKaiju e InventarioDao; InventarioRepository; InventarioViewModelFactory</x:v>
       </x:c>
       <x:c r="E24" s="10" t="str">
-        <x:v>PersistenciaViewModelTest (reabrir); InventarioDaoTest (en teléfono); pauta docs/17 paso 19</x:v>
+        <x:v>PersistenciaViewModelTest (reabrir); InventarioDaoTest (3/3 en emulador); captura 26 de docs/evidencia/capturas</x:v>
       </x:c>
       <x:c r="F24" s="10" t="str">
         <x:v>IE 2.3.1</x:v>

</xml_diff>